<commit_message>
Prepare ATK-Pro v3.0.1 RC1
</commit_message>
<xml_diff>
--- a/docs_generali/Matrice_portali.xlsx
+++ b/docs_generali/Matrice_portali.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrice portali esistenti" sheetId="1" r:id="R74293ec425ac473e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrice portali candidati" sheetId="2" r:id="R70264843059648eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrice portali esistenti" sheetId="1" r:id="Rf4a02dee58de47a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrice portali candidati" sheetId="2" r:id="Re954a49c67f74d55"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -469,7 +469,7 @@
         <x:v>Supportare solo risorse pubbliche/no-login e verificare condizioni del singolo ente</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="132" hidden="0" customHeight="1">
+    <x:row r="8" ht="211.1999969482422" hidden="0" customHeight="1">
       <x:c r="A8" s="10" t="str">
         <x:v>biblioteca_digitale_siena</x:v>
       </x:c>
@@ -492,7 +492,7 @@
         <x:v>Supportare solo manifest item-level pubblici BDS, con range esplicito, ritmo prudente e verifica delle condizioni del singolo oggetto</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="198" hidden="0" customHeight="1">
+    <x:row r="9" ht="132" hidden="0" customHeight="1">
       <x:c r="A9" s="10" t="str">
         <x:v>bub_digitale</x:v>
       </x:c>
@@ -561,7 +561,7 @@
         <x:v>Supportare solo manifest item-level pubblici, evitare collection di annata, usare range esplicito e controllo diritti/licenza del record</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="224.39999389648438" hidden="0" customHeight="1">
+    <x:row r="12" ht="184.8000030517578" hidden="0" customHeight="1">
       <x:c r="A12" s="10" t="str">
         <x:v>phaidra_unipd</x:v>
       </x:c>
@@ -584,7 +584,7 @@
         <x:v>Supportare solo manifest item-level pubblici, con range esplicito e verifica obbligatoria di rights notice/licenza del singolo oggetto</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="211.1999969482422" hidden="0" customHeight="1">
+    <x:row r="13" ht="198" hidden="0" customHeight="1">
       <x:c r="A13" s="10" t="str">
         <x:v>biblioteca_digitale_trentina</x:v>
       </x:c>
@@ -607,7 +607,7 @@
         <x:v>Supporto tecnico su immagini pubbliche; quando l'utente richiede solo PDF e non imposta range, usare il PDF diretto ufficiale</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="145.1999969482422" hidden="0" customHeight="1">
+    <x:row r="14" ht="224.39999389648438" hidden="0" customHeight="1">
       <x:c r="A14" s="10" t="str">
         <x:v>biblioteca_digitale_lombarda</x:v>
       </x:c>
@@ -630,7 +630,7 @@
         <x:v>Supportare solo documento singolo PDF da endpoint REST pubblico; niente immagini, registro o sequenze finche IIIF/info.json non risultano stabili</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="145.1999969482422" hidden="0" customHeight="1">
+    <x:row r="15" ht="211.1999969482422" hidden="0" customHeight="1">
       <x:c r="A15" s="10" t="str">
         <x:v>rovereto_digital_library</x:v>
       </x:c>
@@ -653,7 +653,7 @@
         <x:v>Supportare solo bitstream classificati come pagine iiifpdf-*.png, con range esplicito per record e controllo licenza del singolo item</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="145.1999969482422" hidden="0" customHeight="1">
+    <x:row r="16" ht="264" hidden="0" customHeight="1">
       <x:c r="A16" s="10" t="str">
         <x:v>doge_unige</x:v>
       </x:c>
@@ -676,7 +676,7 @@
         <x:v>Supportare solo derivati pubblici IIIF-ALTERNATIVE-LD e PDF IIIF-ALTERNATIVE-DOWNLOAD, con range esplicito; escludere ORIGINAL e bundle IIIF-PDF-* segnati nodownload</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="132" hidden="0" customHeight="1">
+    <x:row r="17" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A17" s="10" t="str">
         <x:v>memooria</x:v>
       </x:c>
@@ -699,7 +699,7 @@
         <x:v>Usare come capability tecnica, non come portale unico: richiedere verifica per ogni istanza</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="171.60000610351562" hidden="0" customHeight="1">
+    <x:row r="18" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A18" s="10" t="str">
         <x:v>vatlib</x:v>
       </x:c>
@@ -722,7 +722,7 @@
         <x:v>Mantenere con avviso forte e senza presentarlo come fonte liberamente riusabile</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="118.80000305175781" hidden="0" customHeight="1">
+    <x:row r="19" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A19" s="10" t="str">
         <x:v>findbuch</x:v>
       </x:c>
@@ -745,7 +745,7 @@
         <x:v>Mantenere solo per risorse pubbliche e range puntuale; non estendere senza termini dell'ente</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="158.39999389648438" hidden="0" customHeight="1">
+    <x:row r="20" ht="132" hidden="0" customHeight="1">
       <x:c r="A20" s="10" t="str">
         <x:v>matricula</x:v>
       </x:c>
@@ -768,7 +768,7 @@
         <x:v>Mantenere con limite non commerciale, no derivati, citazione/link e senza bulk scraping</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="132" hidden="0" customHeight="1">
+    <x:row r="21" ht="171.60000610351562" hidden="0" customHeight="1">
       <x:c r="A21" s="10" t="str">
         <x:v>gallica</x:v>
       </x:c>
@@ -791,7 +791,7 @@
         <x:v>Consolidare con citazione obbligatoria, rispetto del non commerciale e cautela sui partner</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="158.39999389648438" hidden="0" customHeight="1">
+    <x:row r="22" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A22" s="10" t="str">
         <x:v>heidelberg</x:v>
       </x:c>
@@ -814,7 +814,7 @@
         <x:v>Consolidare con credito fonte e controllo licenza per singolo volume</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="145.1999969482422" hidden="0" customHeight="1">
+    <x:row r="23" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A23" s="10" t="str">
         <x:v>bodleian</x:v>
       </x:c>
@@ -837,7 +837,7 @@
         <x:v>Consolidare IIIF con avviso non commerciale, attribuzione e niente re-hosting sistematico immagini</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="171.60000610351562" hidden="0" customHeight="1">
+    <x:row r="24" ht="132" hidden="0" customHeight="1">
       <x:c r="A24" s="10" t="str">
         <x:v>e_rara</x:v>
       </x:c>
@@ -860,7 +860,7 @@
         <x:v>Consolidare con controllo licenza per documento e citazione della fonte</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="132" hidden="0" customHeight="1">
+    <x:row r="25" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A25" s="10" t="str">
         <x:v>e_codices</x:v>
       </x:c>
@@ -883,7 +883,7 @@
         <x:v>Consolidare con citazione obbligatoria e avviso per usi commerciali/pubblicazioni</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="79.19999694824219" hidden="0" customHeight="1">
+    <x:row r="26" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A26" s="10" t="str">
         <x:v>e_manuscripta</x:v>
       </x:c>
@@ -906,72 +906,72 @@
         <x:v>Consolidare con controllo licenza per documento; evitare copia sistematica/re-hosting</x:v>
       </x:c>
     </x:row>
-    <x:row r="27">
-      <x:c r="A27" t="str">
+    <x:row r="27" ht="171.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A27" s="10" t="str">
         <x:v>internet_archive</x:v>
       </x:c>
-      <x:c r="B27" t="str">
+      <x:c r="B27" s="10" t="str">
         <x:v>Internet Archive</x:v>
       </x:c>
-      <x:c r="C27" t="str">
+      <x:c r="C27" s="10" t="str">
         <x:v>Internazionale</x:v>
       </x:c>
-      <x:c r="D27" t="str">
+      <x:c r="D27" s="10" t="str">
         <x:v>Manifest sintetico da metadata/files/BookReaderImages</x:v>
       </x:c>
-      <x:c r="E27" t="str">
+      <x:c r="E27" s="10" t="str">
         <x:v>Medio-Alto</x:v>
       </x:c>
-      <x:c r="F27" t="str">
+      <x:c r="F27" s="10" t="str">
         <x:v>Licenza e disponibilita variabili per item; alcuni item sono prestito o no-download</x:v>
       </x:c>
-      <x:c r="G27" t="str">
+      <x:c r="G27" s="10" t="str">
         <x:v>Supportare solo item pubblici scaricabili, con licenza/diritti chiari e senza aggirare prestito/no-download</x:v>
       </x:c>
     </x:row>
-    <x:row r="28">
-      <x:c r="A28" t="str">
+    <x:row r="28" ht="132" hidden="0" customHeight="1">
+      <x:c r="A28" s="10" t="str">
         <x:v>europeana</x:v>
       </x:c>
-      <x:c r="B28" t="str">
+      <x:c r="B28" s="10" t="str">
         <x:v>Europeana IIIF</x:v>
       </x:c>
-      <x:c r="C28" t="str">
+      <x:c r="C28" s="10" t="str">
         <x:v>Internazionale</x:v>
       </x:c>
-      <x:c r="D28" t="str">
+      <x:c r="D28" s="10" t="str">
         <x:v>IIIF diretto da provider/record id</x:v>
       </x:c>
-      <x:c r="E28" t="str">
+      <x:c r="E28" s="10" t="str">
         <x:v>Basso-Medio</x:v>
       </x:c>
-      <x:c r="F28" t="str">
+      <x:c r="F28" s="10" t="str">
         <x:v>Diritti da leggere per record/provider; API soggetta a chiave, termini e limiti</x:v>
       </x:c>
-      <x:c r="G28" t="str">
+      <x:c r="G28" s="10" t="str">
         <x:v>Usare solo record con IIIF disponibile, rights statement chiaro e attribution ai provider</x:v>
       </x:c>
     </x:row>
-    <x:row r="29">
-      <x:c r="A29" t="str">
+    <x:row r="29" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A29" s="10" t="str">
         <x:v>manifest_diretto</x:v>
       </x:c>
-      <x:c r="B29" t="str">
+      <x:c r="B29" s="10" t="str">
         <x:v>Manifest diretto (URL gia noto)</x:v>
       </x:c>
-      <x:c r="C29" t="str">
+      <x:c r="C29" s="10" t="str">
         <x:v>Avanzato</x:v>
       </x:c>
-      <x:c r="D29" t="str">
+      <x:c r="D29" s="10" t="str">
         <x:v>URL manifest fornito dall'utente</x:v>
       </x:c>
-      <x:c r="E29" t="str">
+      <x:c r="E29" s="10" t="str">
         <x:v>Variabile</x:v>
       </x:c>
-      <x:c r="F29" t="str">
+      <x:c r="F29" s="10" t="str">
         <x:v>Responsabilita utente + verifica termini origine</x:v>
       </x:c>
-      <x:c r="G29" t="str">
+      <x:c r="G29" s="10" t="str">
         <x:v>Mantenere con avviso/criteri chiari</x:v>
       </x:c>
     </x:row>
@@ -1016,7 +1016,7 @@
         <x:v>Decisione provvisoria</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="382.79998779296875" hidden="0" customHeight="1">
+    <x:row r="2" ht="976.7999877929688" hidden="0" customHeight="1">
       <x:c r="A2" s="10" t="str">
         <x:v>archivi_nazionali</x:v>
       </x:c>
@@ -1039,7 +1039,7 @@
         <x:v>C - candidato strategico per discovery/link assistito e accesso ai servizi; nessun downloader finche non emergono API/IIIF/endpoint pubblici compatibili</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="488.3999938964844" hidden="0" customHeight="1">
+    <x:row r="3" ht="765.5999755859375" hidden="0" customHeight="1">
       <x:c r="A3" s="10" t="str">
         <x:v>archivio_digitale_icar</x:v>
       </x:c>
@@ -1062,7 +1062,7 @@
         <x:v>C - link/discovery assistito e consultazione pubblica; vietare builder/downloader e live smoke di download salvo futuro endpoint ufficiale documentato e autorizzato</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="528" hidden="0" customHeight="1">
+    <x:row r="4" ht="673.2000122070312" hidden="0" customHeight="1">
       <x:c r="A4" s="10" t="str">
         <x:v>sias</x:v>
       </x:c>
@@ -1085,7 +1085,7 @@
         <x:v>C - discovery/link assistito e apertura inventari; no download immagini o PDF massivo senza endpoint e termini specifici</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="475.20001220703125" hidden="0" customHeight="1">
+    <x:row r="5" ht="871.2000122070312" hidden="0" customHeight="1">
       <x:c r="A5" s="10" t="str">
         <x:v>san_risorse_digitali</x:v>
       </x:c>
@@ -1108,7 +1108,7 @@
         <x:v>B - capability futura metadata/OAI piu' concreta; no downloader immagini diretto via SAN</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="462" hidden="0" customHeight="1">
+    <x:row r="6" ht="633.5999755859375" hidden="0" customHeight="1">
       <x:c r="A6" s="10" t="str">
         <x:v>siusa</x:v>
       </x:c>
@@ -1131,7 +1131,7 @@
         <x:v>C - discovery, schede e link assistito; eventuale metadata solo via SAN/open data, nessun downloader</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="660" hidden="0" customHeight="1">
+    <x:row r="7" ht="1016.4000244140625" hidden="0" customHeight="1">
       <x:c r="A7" s="10" t="str">
         <x:v>beweb</x:v>
       </x:c>
@@ -1154,7 +1154,7 @@
         <x:v>C - discovery/link assistito e, al massimo, futura metadata/search su dati catalografici compatibili; no downloader generico</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="541.2000122070312" hidden="0" customHeight="1">
+    <x:row r="8" ht="1016.4000244140625" hidden="0" customHeight="1">
       <x:c r="A8" s="10" t="str">
         <x:v>archivi_diocesani_italiani</x:v>
       </x:c>
@@ -1177,9 +1177,9 @@
         <x:v>C - mappa/link assistiti e schede di orientamento; vietare automazioni generiche, login, aree riservate e download senza fonte pubblica no-login con termini chiari</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="712.7999877929688" hidden="0" customHeight="1">
+    <x:row r="9" ht="607.2000122070312" hidden="0" customHeight="1">
       <x:c r="A9" s="10" t="str">
-        <x:v>archivio_stato_ticino / servizio_archivi_locali_ticino</x:v>
+        <x:v>asti_scopearchiv / asti_mappe_catastali / asti_fondi_fotografici / asti_pergamene</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
         <x:v>Archivio di Stato del Cantone Ticino / SAL</x:v>
@@ -1188,19 +1188,19 @@
         <x:v>Svizzera italiana</x:v>
       </x:c>
       <x:c r="D9" s="10" t="str">
-        <x:v>https://www4.ti.ch/decs/dcsu/asti/servizi/servizio-archivi-locali-sal/; https://www4.ti.ch/fileadmin/DECS/DCSU/ASTI/Documenti/Ricerche_genealogiche.pdf; https://www4.ti.ch/decs/dcsu/asti/servizi/consultazione-e-riproduzione-dei-documenti/; catalogo https://www.archiviodistato.ti.ch/Query/volltextsuche.aspx</x:v>
+        <x:v>https://www4.ti.ch/decs/dcsu/asti/; catalogo https://www.archiviodistato.ti.ch/Query/volltextsuche.aspx; nota tecnica candidati_svizzeri_prossima_release_SAG_ASTi.md</x:v>
       </x:c>
       <x:c r="E9" s="10" t="str">
-        <x:v>Molto alta per Ticino: fondi genealogici 1750-1960, archivi comunali, patriziali e parrocchiali, ruoli di popolazione, stato civile e microfilm ecclesiastici</x:v>
+        <x:v>Molto alta per Ticino: fondi genealogici, archivi comunali e parrocchiali, mappe catastali, fotografie e pergamene</x:v>
       </x:c>
       <x:c r="F9" s="10" t="str">
-        <x:v>Controllo 2026-06-05 + ricontrollo ufficiale 2026-07-31: ASTi/SAL continua a censire e riordinare archivi locali, compresi archivi parrocchiali, e offre strumenti online reali come il catalogo scopeArchiv. La consultazione in sede o in versione digitale resta gratuita, ma regolamento e tariffario confermano emolumenti per alcuni servizi, comprese riproduzioni digitali e supporti di ricerca approfonditi. Le ricerche genealogiche restano soggette a condizioni particolari e a richieste puntuali via formulario; i registri parrocchiali ticinesi risultano ancora accessibili soprattutto tramite FamilySearch o microfilm presso l'Archivio diocesano di Lugano, non come endpoint pubblico ASTi</x:v>
+        <x:v>Verifica 2026-09-27: il perimetro non e' omogeneo. scopeArchiv e pergamene sono soprattutto discovery; le mappe catastali espongono immagini Zoomify recuperabili con selezione esplicita; i fondi fotografici richiedono ancora sonda endpoint e verifica diritti. Ruoli, stato civile e registri parrocchiali restano soggetti a condizioni particolari e non costituiscono un corpus pubblico scaricabile</x:v>
       </x:c>
       <x:c r="G9" s="10" t="str">
-        <x:v>C - link/manuale e schede di orientamento; no downloader ATK-Pro</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="369.6000061035156" hidden="0" customHeight="1">
+        <x:v>B per asti_mappe_catastali con R_LIMITED; REVIEW per fotografie; C discovery per scopeArchiv e pergamene</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="712.7999877929688" hidden="0" customHeight="1">
       <x:c r="A10" s="10" t="str">
         <x:v>archivio_diocesano_lugano</x:v>
       </x:c>
@@ -1223,647 +1223,670 @@
         <x:v>C - solo contatto/link assistito e istruzioni di consultazione</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="686.4000244140625" hidden="0" customHeight="1">
+    <x:row r="11" ht="501.6000061035156" hidden="0" customHeight="1">
       <x:c r="A11" s="10" t="str">
-        <x:v>archivio_stato_grigioni</x:v>
+        <x:v>sag_cmi_ais</x:v>
       </x:c>
       <x:c r="B11" s="10" t="str">
-        <x:v>Archivio di Stato dei Grigioni</x:v>
+        <x:v>Archivio di Stato dei Grigioni (SAG)</x:v>
       </x:c>
       <x:c r="C11" s="10" t="str">
         <x:v>Grigioni italofoni / area retica</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
-        <x:v>https://www.gr.ch/IT/istituzioni/amministrazione/ekud/afk/sag/servizi/fondi/familienforschung/Seiten/default.aspx; https://www.gr.ch/IT/istituzioni/amministrazione/ekud/afk/sag/servizi/fondi/Seiten/default.aspx; https://www.gr.ch/IT/istituzioni/amministrazione/ekud/afk/sag/chisiamo/Seiten/default.aspx</x:v>
+        <x:v>catalogo CMI AIS e nota tecnica candidati_svizzeri_prossima_release_SAG_ASTi.md; https://www.gr.ch/IT/istituzioni/amministrazione/ekud/afk/sag/</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
-        <x:v>Molto alta per valli italofone, mobilita alpina e fonti pre-1876: registri parrocchiali, stato civile, registri dei cittadini, schede genealogiche e strumenti di ricerca</x:v>
+        <x:v>Molto alta per valli italofone, mobilita alpina e fonti pre-1876: registri parrocchiali, stato civile, registri dei cittadini e microfilm</x:v>
       </x:c>
       <x:c r="F11" s="10" t="str">
-        <x:v>Controllo 2026-06-05 + ricontrollo ufficiale 2026-07-31: l'Archivio di Stato conferma che tutti i registri parrocchiali noti sono stati microfilmati e consultabili presso l'Archivio; i registri di stato civile fino al 1929 sono consultabili in sala di lettura, quelli dei cittadini attinenti fino al 1929 su microfilm, mentre i registri delle famiglie dal 1929 non sono visionabili. Il quadro online e' piu' ricco di quanto sembrasse: oltre a PDF e sistema informativo, il sito indica fondi digitalizzati consultabili online e integrazione con Archives Online per metadati e documenti delle banche dati collegate. Resta comunque un ramo soprattutto consultativo e regolato</x:v>
+        <x:v>Verifica pratica 2026-09-27: le API pubbliche CMI AIS consentono ricerca e dettaglio; per numerosi record liberamente accessibili e' disponibile il PDF originale senza login. L'adapter deve rispettare lo stato di accesso item-level, usare streaming, limiti e nomi sicuri e non estendere il download ai record protetti</x:v>
       </x:c>
       <x:c r="G11" s="10" t="str">
-        <x:v>C - discovery/link assistito; no download generale, salvo eventuali fondi digitalizzati con condizioni specifiche</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="435.6000061035156" hidden="0" customHeight="1">
+        <x:v>A - adapter sag_cmi_ais, politica iniziale D_ONLY, priorita' della prossima release funzionale</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="712.7999877929688" hidden="0" customHeight="1">
       <x:c r="A12" s="10" t="str">
+        <x:v>biblioteca_cremona_filestation</x:v>
+      </x:c>
+      <x:c r="B12" s="10" t="str">
+        <x:v>Biblioteca Statale di Cremona - raccolte digitali File Station</x:v>
+      </x:c>
+      <x:c r="C12" s="10" t="str">
+        <x:v>Lombardia / stampa e raccolte locali</x:v>
+      </x:c>
+      <x:c r="D12" s="10" t="str">
+        <x:v>https://bibliocremona.it/patrimonio/biblioteca-digitale/risorse-elettroniche/la-provincia-1883-1923/; https://bibliocremona.it/patrimonio/biblioteca-digitale/; nota tecnica prossima_release_AI_e_Biblioteca_Cremona.md</x:v>
+      </x:c>
+      <x:c r="E12" s="10" t="str">
+        <x:v>Alta: quotidiani storici, materiali digitalizzati e risorse accessibili, con JPEG, PDF e XML strutturato</x:v>
+      </x:c>
+      <x:c r="F12" s="10" t="str">
+        <x:v>Verifica pratica 2026-09-27: API Synology File Station e quattro condivisioni leggibili (LA PROVINCIA, IL REGIME FASCISTA, MATERIALE DIGITALIZZATO, LIS). Un solo connettore puo' esporre quattro profili; le altre risorse del sito richiedono analisi separate. Bloccanti: endpoint IP con certificato non valido per il nome host, credenziali pubbliche soggette a rotazione e condizioni di automazione, attribuzione e riuso non ancora esplicite</x:v>
+      </x:c>
+      <x:c r="G12" s="10" t="str">
+        <x:v>B / HOLD - famiglia synology_file_station, politica proposta R_LIMITED; implementare solo dopo TLS valido e conferma scritta</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="739.2000122070312" hidden="0" customHeight="1">
+      <x:c r="A13" s="10" t="str">
         <x:v>diocesi_chur_coira</x:v>
       </x:c>
-      <x:c r="B12" s="10" t="str">
+      <x:c r="B13" s="10" t="str">
         <x:v>Archivio vescovile di Coira / Bischöfliches Archiv Chur</x:v>
       </x:c>
-      <x:c r="C12" s="10" t="str">
+      <x:c r="C13" s="10" t="str">
         <x:v>Grigioni / area retica ecclesiastica</x:v>
       </x:c>
-      <x:c r="D12" s="10" t="str">
+      <x:c r="D13" s="10" t="str">
         <x:v>https://www.archiv-bistum-chur.ch/; https://www.bistumsarchiv-chur.findbuch.net/; contatti https://www.archiv-bistum-chur.ch/Kontakt.htm</x:v>
       </x:c>
-      <x:c r="E12" s="10" t="str">
+      <x:c r="E13" s="10" t="str">
         <x:v>Alta: diocesi storica antica, rilevante per fonti ecclesiastiche grigionesi e area retica</x:v>
       </x:c>
-      <x:c r="F12" s="10" t="str">
+      <x:c r="F13" s="10" t="str">
         <x:v>Ricontrollo ufficiale 2026-07-31: il sito documenta un archivio ecclesiastico strutturato, con ordinamento dei fondi, repertori online, Findbuch e lavori di digitalizzazione/descrizione in corso su varie serie. La pagina contatti esplicita pero' che il BAC non e' un archivio pubblico: la consultazione e' solo previa richiesta, nel locale di lettura/lavoro e secondo un regolamento proprio. Non emerge quindi una policy di download immagini/API generalizzabile</x:v>
       </x:c>
-      <x:c r="G12" s="10" t="str">
+      <x:c r="G13" s="10" t="str">
         <x:v>C - link/discovery assistito; non estendere come downloader generico</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="396" hidden="0" customHeight="1">
-      <x:c r="A13" s="10" t="str">
+    <x:row r="14" ht="396" hidden="0" customHeight="1">
+      <x:c r="A14" s="10" t="str">
         <x:v>biblioteca_digitale_siena</x:v>
       </x:c>
-      <x:c r="B13" s="10" t="str">
+      <x:c r="B14" s="10" t="str">
         <x:v>Biblioteca Digitale Siena</x:v>
       </x:c>
-      <x:c r="C13" s="10" t="str">
+      <x:c r="C14" s="10" t="str">
         <x:v>Italia</x:v>
       </x:c>
-      <x:c r="D13" s="10" t="str">
+      <x:c r="D14" s="10" t="str">
         <x:v>https://bds.comune.siena.it/; https://bds.comune.siena.it/it/169/</x:v>
       </x:c>
-      <x:c r="E13" s="10" t="str">
+      <x:c r="E14" s="10" t="str">
         <x:v>Media-alta: manoscritti, periodici, disegni, archivi e carteggi senesi/toscani</x:v>
       </x:c>
-      <x:c r="F13" s="10" t="str">
+      <x:c r="F14" s="10" t="str">
         <x:v>Piattaforma pubblica IIIF; termini ufficiali consentono JPG web-resolution per uso personale, studio e ricerca con citazione, vietando uso commerciale e trasformazioni non autorizzate; smoke live 2026-06-05 passato su manifest da 106 canvas</x:v>
       </x:c>
-      <x:c r="G13" s="10" t="str">
+      <x:c r="G14" s="10" t="str">
         <x:v>A - builder viewer-&gt;manifest aggiunto e verificato live</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="448.79998779296875" hidden="0" customHeight="1">
-      <x:c r="A14" s="10" t="str">
+    <x:row r="15" ht="448.79998779296875" hidden="0" customHeight="1">
+      <x:c r="A15" s="10" t="str">
         <x:v>biblioteca_digitale_trentina</x:v>
       </x:c>
-      <x:c r="B14" s="10" t="str">
+      <x:c r="B15" s="10" t="str">
         <x:v>Biblioteca Digitale Trentina</x:v>
       </x:c>
-      <x:c r="C14" s="10" t="str">
+      <x:c r="C15" s="10" t="str">
         <x:v>Italia / Trentino e area ex asburgica</x:v>
       </x:c>
-      <x:c r="D14" s="10" t="str">
+      <x:c r="D15" s="10" t="str">
         <x:v>https://bdt.bibcom.trento.it/; https://bdt.bibcom.trento.it/Riuso; https://www.comune.trento.it/Servizi/Biblioteca-Digitale-Trentina-BDT</x:v>
       </x:c>
-      <x:c r="E14" s="10" t="str">
+      <x:c r="E15" s="10" t="str">
         <x:v>Alta per storia locale, Trentino, mobilita alpina, cartoline, periodici, carte geografiche, stampe e fonti bibliografiche di contesto</x:v>
       </x:c>
-      <x:c r="F14" s="10" t="str">
+      <x:c r="F15" s="10" t="str">
         <x:v>Controllo 2026-06-06: fonte istituzionale pubblica, accesso libero, download gratuito delle immagini e pagina di riuso molto favorevole: materiali in pubblico dominio, riuso anche commerciale con citazione. La sonda ha trovato immagini dirette e PDF diretto, non manifest IIIF reale</x:v>
       </x:c>
-      <x:c r="G14" s="10" t="str">
+      <x:c r="G15" s="10" t="str">
         <x:v>A - promosso a supporto tecnico: manifest sintetico da immagini pubbliche e PDF diretto ufficiale per testi a stampa quando l'utente richiede solo PDF senza range</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="831.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A15" s="10" t="str">
+    <x:row r="16" ht="1095.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A16" s="10" t="str">
         <x:v>beic_digitale</x:v>
       </x:c>
-      <x:c r="B15" s="10" t="str">
+      <x:c r="B16" s="10" t="str">
         <x:v>BEIC digital library</x:v>
-      </x:c>
-      <x:c r="C15" s="10" t="str">
-        <x:v>Italia / Lombardia</x:v>
-      </x:c>
-      <x:c r="D15" s="10" t="str">
-        <x:v>https://digital.beic.it/; https://digital.beic.it/termini-duso/; https://digital.beic.it/infrastruttura-e-standard/; esempi tecnici Preserver https://preserver.beic.it/delivery/DeliveryManagerServlet?dps_pid=IE7400509</x:v>
-      </x:c>
-      <x:c r="E15" s="10" t="str">
-        <x:v>Alta per libri antichi, manoscritti, periodici, editoria lombarda e fonti bibliografiche utili alla ricerca genealogica e territoriale</x:v>
-      </x:c>
-      <x:c r="F15" s="10" t="str">
-        <x:v>Controllo 2026-06-08 + ricontrollo 2026-07-29: termini ufficiali molto favorevoli per opere in pubblico dominio, immagini scaricabili/riutilizzabili e dati CC0; infrastruttura Rosetta/Alma/Primo VE con OAI-PMH documentato. Lato download non e ancora emerso un endpoint utilizzabile in modo ripetibile: il test live su Preserver IE7400509 continua a mostrare solo viewer e logo del sito, mentre il record Primo alma9925210904741 non espone manifest, PDF o immagini utili alla sonda. Il probe ora separa esplicitamente gli asset grafici di sito dai segnali tecnici riusabili e classifica entrambi i campioni come GO/NO-GO: HOLD. verify_beic_technical_probe.py resta lo strumento di raccolta campioni, ma senza integrazione nel menu</x:v>
-      </x:c>
-      <x:c r="G15" s="10" t="str">
-        <x:v>B/C - candidato forte per metadata e valore culturale, ma downloader sospeso finche non emergono campioni BEIC diretti con endpoint file/manifest stabile e policy item-level</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="660" hidden="0" customHeight="1">
-      <x:c r="A16" s="10" t="str">
-        <x:v>biblioteca_digitale_lombarda</x:v>
-      </x:c>
-      <x:c r="B16" s="10" t="str">
-        <x:v>Biblioteca Digitale Lombarda</x:v>
       </x:c>
       <x:c r="C16" s="10" t="str">
         <x:v>Italia / Lombardia</x:v>
       </x:c>
       <x:c r="D16" s="10" t="str">
+        <x:v>https://digital.beic.it/; https://digital.beic.it/termini-duso/; https://digital.beic.it/infrastruttura-e-standard/; esempi tecnici Preserver https://preserver.beic.it/delivery/DeliveryManagerServlet?dps_pid=IE7400509</x:v>
+      </x:c>
+      <x:c r="E16" s="10" t="str">
+        <x:v>Alta per libri antichi, manoscritti, periodici, editoria lombarda e fonti bibliografiche utili alla ricerca genealogica e territoriale</x:v>
+      </x:c>
+      <x:c r="F16" s="10" t="str">
+        <x:v>Controllo 2026-06-08 + ricontrollo 2026-07-29: termini ufficiali molto favorevoli per opere in pubblico dominio, immagini scaricabili/riutilizzabili e dati CC0; infrastruttura Rosetta/Alma/Primo VE con OAI-PMH documentato. Lato download non e ancora emerso un endpoint utilizzabile in modo ripetibile: il test live su Preserver IE7400509 continua a mostrare solo viewer e logo del sito, mentre il record Primo alma9925210904741 non espone manifest, PDF o immagini utili alla sonda. Il probe ora separa esplicitamente gli asset grafici di sito dai segnali tecnici riusabili e classifica entrambi i campioni come GO/NO-GO: HOLD. verify_beic_technical_probe.py resta lo strumento di raccolta campioni, ma senza integrazione nel menu</x:v>
+      </x:c>
+      <x:c r="G16" s="10" t="str">
+        <x:v>B/C - candidato forte per metadata e valore culturale, ma downloader sospeso finche non emergono campioni BEIC diretti con endpoint file/manifest stabile e policy item-level</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="660" hidden="0" customHeight="1">
+      <x:c r="A17" s="10" t="str">
+        <x:v>biblioteca_digitale_lombarda</x:v>
+      </x:c>
+      <x:c r="B17" s="10" t="str">
+        <x:v>Biblioteca Digitale Lombarda</x:v>
+      </x:c>
+      <x:c r="C17" s="10" t="str">
+        <x:v>Italia / Lombardia</x:v>
+      </x:c>
+      <x:c r="D17" s="10" t="str">
         <x:v>https://www.bdl.servizirl.it/; esempi record pubblici https://www.bdl.servizirl.it/vufind/Record/BDL-OGGETTO-133442; endpoint PDF pubblici https://www.bdl.servizirl.it/bdl/public/rest/srv/item/12404/pdf</x:v>
       </x:c>
-      <x:c r="E16" s="10" t="str">
+      <x:c r="E17" s="10" t="str">
         <x:v>Alta per storia locale lombarda, periodici, monografie, archivi e fondi civici</x:v>
       </x:c>
-      <x:c r="F16" s="10" t="str">
+      <x:c r="F17" s="10" t="str">
         <x:v>Controllo 2026-06-08: portale pubblico VuFind con record e PDF REST pubblici; il campione item/12404/pdf risponde come PDF reale ed e promosso a supporto puntuale D_ONLY. La pagina record espone anche una miniatura Cantaloupe/IIIF (6823693) ma insieme ad asset grafici del sito; l'info.json derivato ha dato timeout nel test live. Molti record dichiarano CC BY-NC-ND, quindi uso studio/ricerca con limiti non commerciale/no-derivati</x:v>
       </x:c>
-      <x:c r="G16" s="10" t="str">
+      <x:c r="G17" s="10" t="str">
         <x:v>A/B - promosso solo per PDF puntuale pubblico; niente supporto immagini/registro finche info.json, sequenze o manifest non risultano stabili</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="976.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A17" s="10" t="str">
+    <x:row r="18" ht="976.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A18" s="10" t="str">
         <x:v>ambrosiana_digitale</x:v>
       </x:c>
-      <x:c r="B17" s="10" t="str">
+      <x:c r="B18" s="10" t="str">
         <x:v>Veneranda Biblioteca Ambrosiana - Digital Library</x:v>
       </x:c>
-      <x:c r="C17" s="10" t="str">
+      <x:c r="C18" s="10" t="str">
         <x:v>Italia / Lombardia ecclesiastica e manoscritti</x:v>
       </x:c>
-      <x:c r="D17" s="10" t="str">
+      <x:c r="D18" s="10" t="str">
         <x:v>https://www.ambrosiana.it/en/discover/masterpieces/the-digital-library/; https://ambrosiana.comperio.it/library-digital/; esempi Comperio https://ambrosiana.comperio.it/opac/detail/view/ambro:catalog:24203; campione pubblico UniCatt/Veneranda https://digitallibrary.unicatt.it/veneranda/data/public/manifests/0b/02/da/82/80/0d/10/a0/0b02da82800d10a0.json</x:v>
       </x:c>
-      <x:c r="E17" s="10" t="str">
+      <x:c r="E18" s="10" t="str">
         <x:v>Alta per manoscritti, codici, fondi storici e fonti culturali collegate a Milano e Lombardia</x:v>
       </x:c>
-      <x:c r="F17" s="10" t="str">
+      <x:c r="F18" s="10" t="str">
         <x:v>Controllo 2026-06-07/2026-07-25: la pagina ufficiale descrive accesso libero e uso dello standard IIIF; fonte accademica conferma Mirador e Cantaloupe. Test live su ambro:catalog:24203: trovati solo record Comperio duplicati/correlati e asset grafico, nessun manifest, info.json, immagine Cantaloupe o viewer utile. Verifica aggiuntiva su piattaforma pubblica UniCatt/Veneranda: manifest IIIF scaricato con codice 200 e 101 canvas. La pista tecnica esiste quindi davvero, ma la UI pubblica segnala No Downloadable; senza termini item-level compatibili o autorizzazione esplicita al download, il ramo resta fuori dal downloader</x:v>
       </x:c>
-      <x:c r="G17" s="10" t="str">
+      <x:c r="G18" s="10" t="str">
         <x:v>B/C - valore alto e IIIF pubblico confermato, ma integrazione sospesa per restrizione No Downloadable e assenza di termini item-level che autorizzino il download</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="858" hidden="0" customHeight="1">
-      <x:c r="A18" s="10" t="str">
+    <x:row r="19" ht="858" hidden="0" customHeight="1">
+      <x:c r="A19" s="10" t="str">
         <x:v>rovereto_digital_library</x:v>
       </x:c>
-      <x:c r="B18" s="10" t="str">
+      <x:c r="B19" s="10" t="str">
         <x:v>Rovereto Digital Library / Biblioteca Tartarotti</x:v>
       </x:c>
-      <x:c r="C18" s="10" t="str">
+      <x:c r="C19" s="10" t="str">
         <x:v>Italia / Trentino</x:v>
       </x:c>
-      <x:c r="D18" s="10" t="str">
+      <x:c r="D19" s="10" t="str">
         <x:v>https://digitallibrary.bibliotecacivica.rovereto.tn.it/; campioni https://digitallibrary.bibliotecacivica.rovereto.tn.it/entities/publication/e4199e9b-c79b-4c3d-b157-be2dcfc0407f, https://digitallibrary.bibliotecacivica.rovereto.tn.it/entities/picture/2cbeaeab-833a-48c2-9b39-29484ed1c681; termini https://digitallibrary.bibliotecacivica.rovereto.tn.it/info/end-user-agreement</x:v>
       </x:c>
-      <x:c r="E18" s="10" t="str">
+      <x:c r="E19" s="10" t="str">
         <x:v>Media-alta per storia locale trentina, fotografie, documenti d'archivio, riviste e contesto familiare</x:v>
       </x:c>
-      <x:c r="F18" s="10" t="str">
+      <x:c r="F19" s="10" t="str">
         <x:v>Controllo 2026-06-08: portale operativo DSpace-GLAM promosso a supporto tecnico prudente. ATK-Pro deriva l'endpoint REST item standard, segue la paginazione HAL/JSON di bundle e bitstream, costruisce un manifest sintetico solo dai bitstream pubblici classificati come pagine iiifpdf-*.png e conserva il PDF originale solo come riferimento seeAlso. Restano esclusi licenza, miniature/cover e derivati testuali/OCR. Termini ufficiali: accesso libero e gratuito ai file digitali in risoluzione web secondo licenze specifiche; alta definizione su richiesta</x:v>
       </x:c>
-      <x:c r="G18" s="10" t="str">
+      <x:c r="G19" s="10" t="str">
         <x:v>A - promosso a supporto tecnico R_LIMITED con range esplicito e controllo licenza item-level</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="937.2000122070312" hidden="0" customHeight="1">
-      <x:c r="A19" s="10" t="str">
+    <x:row r="20" ht="937.2000122070312" hidden="0" customHeight="1">
+      <x:c r="A20" s="10" t="str">
         <x:v>bub_digitale</x:v>
       </x:c>
-      <x:c r="B19" s="10" t="str">
+      <x:c r="B20" s="10" t="str">
         <x:v>BUB Digitale / Biblioteca Universitaria di Bologna</x:v>
-      </x:c>
-      <x:c r="C19" s="10" t="str">
-        <x:v>Italia / Emilia-Romagna</x:v>
-      </x:c>
-      <x:c r="D19" s="10" t="str">
-        <x:v>https://bub.unibo.it/it/bub-digitale; https://bub.unibo.it/it/bub-digitale/bollettini-parrocchiali; campioni Bondanello 1934 e Castenaso 1933</x:v>
-      </x:c>
-      <x:c r="E19" s="10" t="str">
-        <x:v>Media-alta: papiri, manoscritti greci/arabi/ebraici, opere a stampa, periodici storici, bollettini parrocchiali, fotografie e fondi bolognesi utili al contesto storico-familiare</x:v>
-      </x:c>
-      <x:c r="F19" s="10" t="str">
-        <x:v>Controllo 2026-06-08: fonte ufficiale BUB descrive accesso libero e gratuito per studio/ricerca, uso dello standard IIIF e visualizzatore Mirador. La landing page live espone soprattutto pagine del portale e immagini Plone @@images, ora classificate come plone_page_image per non confonderle con pagine documento. Test live mirato sul bollettino Bondanello 1934: manifest IIIF v2 pulito da viewer_manifest_parameter, codice 200, 44 canvas. Secondo campione Castenaso 1933: manifest diretto, codice 200, 32 canvas. Pattern manifest stabile su piu bollettini; promosso a supporto IIIF diretto prudente</x:v>
-      </x:c>
-      <x:c r="G19" s="10" t="str">
-        <x:v>A - promosso a supporto R_LIMITED: solo manifest BUB pubblici, range esplicito, referer BUB e verifica licenza item-level</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="871.2000122070312" hidden="0" customHeight="1">
-      <x:c r="A20" s="10" t="str">
-        <x:v>dl_ficlit</x:v>
-      </x:c>
-      <x:c r="B20" s="10" t="str">
-        <x:v>FICLIT Digital Library / Universita di Bologna</x:v>
       </x:c>
       <x:c r="C20" s="10" t="str">
         <x:v>Italia / Emilia-Romagna</x:v>
       </x:c>
       <x:c r="D20" s="10" t="str">
+        <x:v>https://bub.unibo.it/it/bub-digitale; https://bub.unibo.it/it/bub-digitale/bollettini-parrocchiali; campioni Bondanello 1934 e Castenaso 1933</x:v>
+      </x:c>
+      <x:c r="E20" s="10" t="str">
+        <x:v>Media-alta: papiri, manoscritti greci/arabi/ebraici, opere a stampa, periodici storici, bollettini parrocchiali, fotografie e fondi bolognesi utili al contesto storico-familiare</x:v>
+      </x:c>
+      <x:c r="F20" s="10" t="str">
+        <x:v>Controllo 2026-06-08: fonte ufficiale BUB descrive accesso libero e gratuito per studio/ricerca, uso dello standard IIIF e visualizzatore Mirador. La landing page live espone soprattutto pagine del portale e immagini Plone @@images, ora classificate come plone_page_image per non confonderle con pagine documento. Test live mirato sul bollettino Bondanello 1934: manifest IIIF v2 pulito da viewer_manifest_parameter, codice 200, 44 canvas. Secondo campione Castenaso 1933: manifest diretto, codice 200, 32 canvas. Pattern manifest stabile su piu bollettini; promosso a supporto IIIF diretto prudente</x:v>
+      </x:c>
+      <x:c r="G20" s="10" t="str">
+        <x:v>A - promosso a supporto R_LIMITED: solo manifest BUB pubblici, range esplicito, referer BUB e verifica licenza item-level</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="871.2000122070312" hidden="0" customHeight="1">
+      <x:c r="A21" s="10" t="str">
+        <x:v>dl_ficlit</x:v>
+      </x:c>
+      <x:c r="B21" s="10" t="str">
+        <x:v>FICLIT Digital Library / Universita di Bologna</x:v>
+      </x:c>
+      <x:c r="C21" s="10" t="str">
+        <x:v>Italia / Emilia-Romagna</x:v>
+      </x:c>
+      <x:c r="D21" s="10" t="str">
         <x:v>https://dl.ficlit.unibo.it/s/lib/page/progetto; campioni https://dl.ficlit.unibo.it/s/lib/item/199245, https://dl.ficlit.unibo.it/s/lib/item/28429</x:v>
       </x:c>
-      <x:c r="E20" s="10" t="str">
+      <x:c r="E21" s="10" t="str">
         <x:v>Media: collezioni accademiche e umanistiche, fonti letterarie, bibliografiche e documentarie utili a ricerche storiche territoriali</x:v>
       </x:c>
-      <x:c r="F20" s="10" t="str">
+      <x:c r="F21" s="10" t="str">
         <x:v>Controllo 2026-06-08: fonte ufficiale descrive piattaforma Omeka S, tecnologia IIIF per immagini e visualizzazione con Mirador Viewer. Test live 2026-06-09: item Corbiere 199245 con immagine originale pubblica e manifest https://dl.ficlit.unibo.it/iiif/2/199245/manifest, codice 200 e 1 canvas; item Camporesi 28429 con immagine originale pubblica e manifest https://dl.ficlit.unibo.it/iiif/2/28429/manifest, codice 200 e 239 canvas. Il pattern Omeka/IIIF appare concreto; restano da verificare termini item set e distinzione tra collezioni liberamente scaricabili e sola consultazione</x:v>
       </x:c>
-      <x:c r="G20" s="10" t="str">
+      <x:c r="G21" s="10" t="str">
         <x:v>A - promosso a supporto tecnico R_LIMITED: solo item/manifest FICLIT pubblici, range esplicito, referer FICLIT e verifica termini item-level</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="1320" hidden="0" customHeight="1">
-      <x:c r="A21" s="10" t="str">
+    <x:row r="22" ht="1584" hidden="0" customHeight="1">
+      <x:c r="A22" s="10" t="str">
         <x:v>impronte_digitali_unifi</x:v>
       </x:c>
-      <x:c r="B21" s="10" t="str">
+      <x:c r="B22" s="10" t="str">
         <x:v>Impronte Digitali / Universita di Firenze</x:v>
       </x:c>
-      <x:c r="C21" s="10" t="str">
+      <x:c r="C22" s="10" t="str">
         <x:v>Italia / Toscana</x:v>
       </x:c>
-      <x:c r="D21" s="10" t="str">
+      <x:c r="D22" s="10" t="str">
         <x:v>https://improntedigitali.unifi.it/; news ufficiale https://www.sba.unifi.it/n2411.html; collezioni digitalizzate https://www.sba.unifi.it/p1308.html; campione https://improntedigitali.unifi.it/items/ea8510d3-4f09-41b6-b69a-5c4ff3d0d082; sonda verify_unifi_technical_probe.py</x:v>
       </x:c>
-      <x:c r="E21" s="10" t="str">
+      <x:c r="E22" s="10" t="str">
         <x:v>Media-alta: periodici, fondi archivistici, materiali rari e di pregio delle biblioteche Unifi, con interesse per contesto storico toscano e universitario</x:v>
       </x:c>
-      <x:c r="F21" s="10" t="str">
+      <x:c r="F22" s="10" t="str">
         <x:v>Controllo 2026-07-26 + ricontrollo 2026-07-29: la fonte ufficiale UniFI descrive il portale come digital library pubblica basata su DSpace-GLAM con viewer Mirador e standard IIIF. Verifica live sull'item Ricordi di architettura (ea8510d3-4f09-41b6-b69a-5c4ff3d0d082): API pubblica server/api/core/items/{uuid} leggibile senza login; bundle pubblici ORIGINAL, LICENSE e MAG; metadati item-level con dc.rights.holder UniFI e dc.rights.license = CC BY-NC-SA; file MAG scaricabile con codice 200; thumbnail generato (THUMBNAIL) accessibile come immagine JPEG pubblica, anche via endpoint item-level /thumbnail. Il ricontrollo del 2026-07-29 amplia il quadro del backend pubblico (record, entity correlate, item API, bundle, bitstream e surrogate, 410 candidati classificati), ma non cambia la sostanza: il primo bitstream immagine del bundle ORIGINAL resta 401 sul content diretto, i metadati del bitstream segnalano bitstream.viewer.provider = iiif insieme a nodownload, e non emergono manifest IIIF pubblici espliciti o info.json riusabili</x:v>
       </x:c>
-      <x:c r="G21" s="10" t="str">
+      <x:c r="G22" s="10" t="str">
         <x:v>B - candidato forte e reale per backend DSpace-GLAM/IIIF, confermato in REVIEW: metadata e surrogate web pubblici si', ma senza download/manifest diretto ancora riusabile</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="514.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A22" s="10" t="str">
+    <x:row r="23" ht="1491.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A23" s="10" t="str">
         <x:v>doge_unige</x:v>
       </x:c>
-      <x:c r="B22" s="10" t="str">
+      <x:c r="B23" s="10" t="str">
         <x:v>DOGE Digital Library / Universita di Genova</x:v>
       </x:c>
-      <x:c r="C22" s="10" t="str">
+      <x:c r="C23" s="10" t="str">
         <x:v>Italia / Liguria</x:v>
       </x:c>
-      <x:c r="D22" s="10" t="str">
+      <x:c r="D23" s="10" t="str">
         <x:v>https://doge.unige.net/; fonti SBA https://biblioteche.unige.it/doge_informazioni_generali, https://biblioteche.unige.it/doge_servizi_offerti; campione https://doge.unige.net/entities/publication/b1c2be2c-e1ae-4676-93e3-07e8e8398f72; sonda verify_doge_technical_probe.py</x:v>
       </x:c>
-      <x:c r="E22" s="10" t="str">
+      <x:c r="E23" s="10" t="str">
         <x:v>Media-alta: libri antichi, materiali scientifici, disegni, fondi storici e patrimonio universitario ligure, utile per contesto storico territoriale e bibliografico</x:v>
       </x:c>
-      <x:c r="F22" s="10" t="str">
+      <x:c r="F23" s="10" t="str">
         <x:v>Controllo 2026-07-26/27: le fonti ufficiali SBA descrivono DOGE come digital library basata su DSpace-GLAM, con Mirador, protocollo IIIF, OAI-PMH e licenza generale CC BY-SA per gli oggetti UniGe, CC0 per i metadati. Verifica live sul campione Euler b1c2be2c-e1ae-4676-93e3-07e8e8398f72: item API pubblico, handle persistente, dc.rights.license = CC BY-SA; bundle ORIGINAL, THUMBNAIL, BRANDED_PREVIEW, IIIF-PDF-*, IIIF-ALTERNATIVE-LD e IIIF-ALTERNATIVE-DOWNLOAD. I contenuti ORIGINAL e IIIF-PDF-* restano bloccati o marcati nodownload, ma i derivati IIIF-ALTERNATIVE-LD risultano pubblici pagina-per-pagina con 373 bitstream JPEG numerati e IIIF-ALTERNATIVE-DOWNLOAD espone un PDF derivato pubblico con codice 200. ATK-Pro ora costruisce quindi un manifest sintetico prudente solo dai derivati IIIF-ALTERNATIVE-LD, con PDF derivato in seeAlso, referer DOGE, range esplicito e senza toccare originali o frame viewer nodownload</x:v>
       </x:c>
-      <x:c r="G22" s="10" t="str">
+      <x:c r="G23" s="10" t="str">
         <x:v>A - promosso a supporto tecnico prudente R_LIMITED: solo derivati pubblici IIIF-ALTERNATIVE-LD + IIIF-ALTERNATIVE-DOWNLOAD, con controllo licenza item-level e divieto di estensione agli originali</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="501.6000061035156" hidden="0" customHeight="1">
-      <x:c r="A23" s="10" t="str">
+    <x:row r="24" ht="1320" hidden="0" customHeight="1">
+      <x:c r="A24" s="10" t="str">
         <x:v>orientales_unior</x:v>
       </x:c>
-      <x:c r="B23" s="10" t="str">
+      <x:c r="B24" s="10" t="str">
         <x:v>OrienTales / Biblioteca digitale Universita di Napoli L'Orientale</x:v>
       </x:c>
-      <x:c r="C23" s="10" t="str">
+      <x:c r="C24" s="10" t="str">
         <x:v>Italia / Campania</x:v>
       </x:c>
-      <x:c r="D23" s="10" t="str">
+      <x:c r="D24" s="10" t="str">
         <x:v>https://www.unior.it/it/biblioteche/servizi-gli-utenti/biblioteca-digitale</x:v>
       </x:c>
-      <x:c r="E23" s="10" t="str">
+      <x:c r="E24" s="10" t="str">
         <x:v>Media-alta: libri antichi, manoscritti in lingue orientali, materiale d'archivio, documentario, periodici, collane, carte geografiche e atlanti, con valore culturale e storico per ricerche italiane</x:v>
       </x:c>
-      <x:c r="F23" s="10" t="str">
+      <x:c r="F24" s="10" t="str">
         <x:v>Controllo 2026-06-08/10: fonte ufficiale indica licenze Creative Commons, framework IIIF, uso di Mirador, download laddove la licenza lo permetta, OCR e scarico metadati; la descrizione tecnica cita DSpace, mentre restano possibili tracce Omeka dai progetti precedenti. verify_orientales_technical_probe.py ora cerca sia pattern DSpace (entities, REST item, bundle, bitstream, handle e link JSON/HAL), sia record Omeka, viewer Mirador, manifest IIIF, info.json, immagini, OCR/testi e metadati candidati. Verifica manuale 2026-06-10: le pagine record finora viste mostrano "Il record non puo essere mostrato agli utenti ospiti" e contenuti riservati agli utenti affiliati; manca quindi il requisito minimo di accesso pubblico senza autenticazione. Il download non e generalizzabile senza record pubblici e licenza dell'oggetto</x:v>
       </x:c>
-      <x:c r="G23" s="10" t="str">
+      <x:c r="G24" s="10" t="str">
         <x:v>C - sospeso/escluso dal download automatico finche non emergono record pubblici consultabili da ospite con licenza visibile e endpoint manifest/bitstream senza autenticazione</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="660" hidden="0" customHeight="1">
-      <x:c r="A24" s="10" t="str">
+    <x:row r="25" ht="514.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A25" s="10" t="str">
         <x:v>museu_imigracao_sp</x:v>
       </x:c>
-      <x:c r="B24" s="10" t="str">
+      <x:c r="B25" s="10" t="str">
         <x:v>Museu da Imigracao do Estado de Sao Paulo - Acervo Digital</x:v>
-      </x:c>
-      <x:c r="C24" s="10" t="str">
-        <x:v>Brasile / diaspora italiana</x:v>
-      </x:c>
-      <x:c r="D24" s="10" t="str">
-        <x:v>https://museudaimigracao.org.br/acervo/sobre-acervo; https://www.museudaimigracao.org.br/acervo/passageiros; https://museudaimigracao.org.br/acervo-e-pesquisa/acervo</x:v>
-      </x:c>
-      <x:c r="E24" s="10" t="str">
-        <x:v>Molto alta per immigrati italiani in Brasile/Sao Paulo</x:v>
-      </x:c>
-      <x:c r="F24" s="10" t="str">
-        <x:v>Acervo digitale pubblico con piu di 250 mila immagini, registri di matricola, liste di bordo, carte di chiamata, richieste SACOP, iconografie, cartografie e giornali; le fonti ufficiali indicano uso/download non commerciale, ma il percorso tecnico appare basato su ricerca web e PDF/immagini pubbliche, non su IIIF/API documentata</x:v>
-      </x:c>
-      <x:c r="G24" s="10" t="str">
-        <x:v>B - candidato forte, ma non integrare finche non viene validata una capability pdf_direct/download diretto pubblica e testabile</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="633.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A25" s="10" t="str">
-        <x:v>apesp_digitalizados</x:v>
-      </x:c>
-      <x:c r="B25" s="10" t="str">
-        <x:v>Arquivo Publico do Estado de Sao Paulo - Acervo digitalizado</x:v>
       </x:c>
       <x:c r="C25" s="10" t="str">
         <x:v>Brasile / diaspora italiana</x:v>
       </x:c>
       <x:c r="D25" s="10" t="str">
-        <x:v>https://web.arquivoestado.sp.gov.br/web/acervo/digitalizados; https://www.arquivoestado.sp.gov.br/web/digitalizado/textual/nucleos_coloniais; https://web.arquivoestado.sp.gov.br/web/acervo/atendimento/reproducao_documentos; https://web.arquivoestado.sp.gov.br/web/acervo/solicitacao_certidoes/imigracao</x:v>
+        <x:v>https://museudaimigracao.org.br/acervo/sobre-acervo; https://www.museudaimigracao.org.br/acervo/passageiros; https://museudaimigracao.org.br/acervo-e-pesquisa/acervo</x:v>
       </x:c>
       <x:c r="E25" s="10" t="str">
-        <x:v>Molto alta: Hospedaria, Porto di Santos, nuclei coloniali, documenti di immigrazione e colonizzazione</x:v>
+        <x:v>Molto alta per immigrati italiani in Brasile/Sao Paulo</x:v>
       </x:c>
       <x:c r="F25" s="10" t="str">
-        <x:v>Fonte ufficiale molto rilevante, ma l'acervo digitalizzato rimanda a registrazione/login e la pagina dei nuclei coloniali contiene avviso di servizio con login; la riproduzione e soggetta a credito, termini di responsabilita e valutazioni su diritto/autorizzazione. Nessun endpoint no-login/API/IIIF stabile verificato nel primo controllo</x:v>
+        <x:v>Acervo digitale pubblico con piu di 250 mila immagini, registri di matricola, liste di bordo, carte di chiamata, richieste SACOP, iconografie, cartografie e giornali; le fonti ufficiali indicano uso/download non commerciale, ma il percorso tecnico appare basato su ricerca web e PDF/immagini pubbliche, non su IIIF/API documentata</x:v>
       </x:c>
       <x:c r="G25" s="10" t="str">
-        <x:v>C - link/manuale e discovery; download diretto escluso finche non emerge una risorsa pubblica no-login con licenza e tecnica stabili</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="607.2000122070312" hidden="0" customHeight="1">
+        <x:v>B - candidato forte, ma non integrare finche non viene validata una capability pdf_direct/download diretto pubblica e testabile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="501.6000061035156" hidden="0" customHeight="1">
       <x:c r="A26" s="10" t="str">
-        <x:v>arquivo_nacional_br_sian</x:v>
+        <x:v>apesp_digitalizados</x:v>
       </x:c>
       <x:c r="B26" s="10" t="str">
-        <x:v>Arquivo Nacional do Brasil / SIAN</x:v>
+        <x:v>Arquivo Publico do Estado de Sao Paulo - Acervo digitalizado</x:v>
       </x:c>
       <x:c r="C26" s="10" t="str">
         <x:v>Brasile / diaspora italiana</x:v>
       </x:c>
       <x:c r="D26" s="10" t="str">
+        <x:v>https://web.arquivoestado.sp.gov.br/web/acervo/digitalizados; https://www.arquivoestado.sp.gov.br/web/digitalizado/textual/nucleos_coloniais; https://web.arquivoestado.sp.gov.br/web/acervo/atendimento/reproducao_documentos; https://web.arquivoestado.sp.gov.br/web/acervo/solicitacao_certidoes/imigracao</x:v>
+      </x:c>
+      <x:c r="E26" s="10" t="str">
+        <x:v>Molto alta: Hospedaria, Porto di Santos, nuclei coloniali, documenti di immigrazione e colonizzazione</x:v>
+      </x:c>
+      <x:c r="F26" s="10" t="str">
+        <x:v>Fonte ufficiale molto rilevante, ma l'acervo digitalizzato rimanda a registrazione/login e la pagina dei nuclei coloniali contiene avviso di servizio con login; la riproduzione e soggetta a credito, termini di responsabilita e valutazioni su diritto/autorizzazione. Nessun endpoint no-login/API/IIIF stabile verificato nel primo controllo</x:v>
+      </x:c>
+      <x:c r="G26" s="10" t="str">
+        <x:v>C - link/manuale e discovery; download diretto escluso finche non emerge una risorsa pubblica no-login con licenza e tecnica stabili</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="660" hidden="0" customHeight="1">
+      <x:c r="A27" s="10" t="str">
+        <x:v>arquivo_nacional_br_sian</x:v>
+      </x:c>
+      <x:c r="B27" s="10" t="str">
+        <x:v>Arquivo Nacional do Brasil / SIAN</x:v>
+      </x:c>
+      <x:c r="C27" s="10" t="str">
+        <x:v>Brasile / diaspora italiana</x:v>
+      </x:c>
+      <x:c r="D27" s="10" t="str">
         <x:v>https://www.gov.br/arquivonacional/pt-br/canais_atendimento/imprensa/copy_of_noticias/a-imigracao-italiana-e-o-acervo-do-an; https://www.gov.br/arquivonacional/pt-br/canais_atendimento/imprensa/copy_of_noticias/quer-pesquisar-no-arquivo-nacional-acesse-o-sian; https://www.gov.br/arquivonacional/pt-br/servicos/acervos/copy_of_acervos-mais-consultados/entrada-de-estrangeiros; https://www.gov.br/arquivonacional/pt-br/servicos/bases-de-dados/bases</x:v>
       </x:c>
-      <x:c r="E26" s="10" t="str">
+      <x:c r="E27" s="10" t="str">
         <x:v>Alta: ingresso di stranieri, vapori, acervo nazionale, Porto di Rio de Janeiro e Porto di Santos</x:v>
       </x:c>
-      <x:c r="F26" s="10" t="str">
+      <x:c r="F27" s="10" t="str">
         <x:v>SIAN e molto rilevante e offre documenti digitalizzati senza costo, ma le fonti ufficiali richiedono cadastro/login; la pagina SIAN espone anche controllo anti-spam/umano. La base separata Entrada de Estrangeiros - Porto do Rio de Janeiro e utile come ricerca nominale/dichiarazione, ma non e ancora un endpoint immagini/API verificato</x:v>
       </x:c>
-      <x:c r="G26" s="10" t="str">
+      <x:c r="G27" s="10" t="str">
         <x:v>C - link/manuale e discovery; non integrare download diretto SIAN per login/challenge. Rivalutare separatamente la base Rio solo se emerge un accesso pubblico documentato e testabile</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="739.2000122070312" hidden="0" customHeight="1">
-      <x:c r="A27" s="10" t="str">
+    <x:row r="28" ht="633.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A28" s="10" t="str">
         <x:v>agn_argentina_inmigrantes</x:v>
       </x:c>
-      <x:c r="B27" s="10" t="str">
+      <x:c r="B28" s="10" t="str">
         <x:v>Archivo General de la Nacion Argentina - buscador inmigrantes</x:v>
-      </x:c>
-      <x:c r="C27" s="10" t="str">
-        <x:v>Argentina / diaspora italiana</x:v>
-      </x:c>
-      <x:c r="D27" s="10" t="str">
-        <x:v>https://www.argentina.gob.ar/interior/archivo-general-de-la-nacion; https://www.argentina.gob.ar/interior/archivo-general-de-la-nacion/consulta-de-antecedentes-migratorios; https://www.argentina.gob.ar/noticias/el-archivo-general-de-la-nacion-es-memoria-del-mundo; https://www.argentina.gob.ar/terminos-y-condiciones; https://www.unesco.org/es/memory-world/lac/passengers-entry-books-sea-1882-1937-national-registry-migrations-documentary-fond</x:v>
-      </x:c>
-      <x:c r="E27" s="10" t="str">
-        <x:v>Molto alta: ingressi al porto di Buenos Aires 1882-1937, serie UNESCO Memoria del Mundo, oltre 4 milioni di ingressi in 808 libri</x:v>
-      </x:c>
-      <x:c r="F27" s="10" t="str">
-        <x:v>Buscador ufficiale pubblico: la pagina indica ricerca per date, nome, cognome e nave, con possibilita di scaricare una constancia PDF e, se digitalizzato, il PDF del libro completo. I termini generali Argentina.gob.ar indicano accesso libero/gratuito e contenuti CC BY 4.0 salvo diversa indicazione; non emergono pero API/IIIF o endpoint ufficiali documentati per automazione</x:v>
-      </x:c>
-      <x:c r="G27" s="10" t="str">
-        <x:v>B - candidato forte per futura capability metadata/PDF; per ora link assistito, no download diretto finche non viene validato un endpoint pubblico stabile con fixture</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="158.39999389648438" hidden="0" customHeight="1">
-      <x:c r="A28" s="10" t="str">
-        <x:v>cemla_buscador</x:v>
-      </x:c>
-      <x:c r="B28" s="10" t="str">
-        <x:v>CEMLA buscador inmigrantes</x:v>
       </x:c>
       <x:c r="C28" s="10" t="str">
         <x:v>Argentina / diaspora italiana</x:v>
       </x:c>
       <x:c r="D28" s="10" t="str">
+        <x:v>https://www.argentina.gob.ar/interior/archivo-general-de-la-nacion; https://www.argentina.gob.ar/interior/archivo-general-de-la-nacion/consulta-de-antecedentes-migratorios; https://www.argentina.gob.ar/noticias/el-archivo-general-de-la-nacion-es-memoria-del-mundo; https://www.argentina.gob.ar/terminos-y-condiciones; https://www.unesco.org/es/memory-world/lac/passengers-entry-books-sea-1882-1937-national-registry-migrations-documentary-fond</x:v>
+      </x:c>
+      <x:c r="E28" s="10" t="str">
+        <x:v>Molto alta: ingressi al porto di Buenos Aires 1882-1937, serie UNESCO Memoria del Mundo, oltre 4 milioni di ingressi in 808 libri</x:v>
+      </x:c>
+      <x:c r="F28" s="10" t="str">
+        <x:v>Buscador ufficiale pubblico: la pagina indica ricerca per date, nome, cognome e nave, con possibilita di scaricare una constancia PDF e, se digitalizzato, il PDF del libro completo. I termini generali Argentina.gob.ar indicano accesso libero/gratuito e contenuti CC BY 4.0 salvo diversa indicazione; non emergono pero API/IIIF o endpoint ufficiali documentati per automazione</x:v>
+      </x:c>
+      <x:c r="G28" s="10" t="str">
+        <x:v>B - candidato forte per futura capability metadata/PDF; per ora link assistito, no download diretto finche non viene validato un endpoint pubblico stabile con fixture</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="607.2000122070312" hidden="0" customHeight="1">
+      <x:c r="A29" s="10" t="str">
+        <x:v>cemla_buscador</x:v>
+      </x:c>
+      <x:c r="B29" s="10" t="str">
+        <x:v>CEMLA buscador inmigrantes</x:v>
+      </x:c>
+      <x:c r="C29" s="10" t="str">
+        <x:v>Argentina / diaspora italiana</x:v>
+      </x:c>
+      <x:c r="D29" s="10" t="str">
         <x:v>https://cemla.com/; https://www.cemla.com/buscador/; https://cemla.com/faqs/; https://cemla.com/contacto/; https://cemla.com/terms-and-conditions/</x:v>
       </x:c>
-      <x:c r="E28" s="10" t="str">
+      <x:c r="E29" s="10" t="str">
         <x:v>Alta: arrivi di immigrati in Argentina, con dati fino al 1960 e forte utilita per famiglie italiane</x:v>
       </x:c>
-      <x:c r="F28" s="10" t="str">
+      <x:c r="F29" s="10" t="str">
         <x:v>Fonte privata/non governativa molto usata; le FAQ chiariscono che CEMLA espone solo i dati presenti nel buscador, indica i campi disponibili e rimanda al certificato via email. Il buscador e incorporato come iframe, non espone API/IIIF o endpoint documentati, la pagina termini e un placeholder generico e il flusso pubblico richiede validazione tipo CAPTCHA</x:v>
       </x:c>
-      <x:c r="G28" s="10" t="str">
+      <x:c r="G29" s="10" t="str">
         <x:v>C - solo link/manuale; no download diretto e no interrogazione automatica senza autorizzazione/API esplicita</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="158.39999389648438" hidden="0" customHeight="1">
-      <x:c r="A29" s="10" t="str">
+    <x:row r="30" ht="739.2000122070312" hidden="0" customHeight="1">
+      <x:c r="A30" s="10" t="str">
         <x:v>agn_colombia_dataviva</x:v>
       </x:c>
-      <x:c r="B29" s="10" t="str">
+      <x:c r="B30" s="10" t="str">
         <x:v>Archivo General de la Nacion Colombia - DataViva</x:v>
       </x:c>
-      <x:c r="C29" s="10" t="str">
+      <x:c r="C30" s="10" t="str">
         <x:v>Colombia / diaspora italiana</x:v>
       </x:c>
-      <x:c r="D29" s="10" t="str">
+      <x:c r="D30" s="10" t="str">
         <x:v>https://www.archivogeneral.gov.co/agn/home/; https://dataviva.archivogeneral.gov.co/; https://www.datos.gov.co/Cultura/DATAVIVA/r5h9-7h58; https://www.archivogeneral.gov.co/dataviva-da-un-paso-historico-hacia-los-datos-abiertos-en-colombia; https://www.archivogeneral.gov.co/terminos-y-condiciones; https://www.archivogeneral.gov.co/sites/default/files/2025-07/MANUAL_DATAVIVA.pdf</x:v>
       </x:c>
-      <x:c r="E29" s="10" t="str">
+      <x:c r="E30" s="10" t="str">
         <x:v>Media-alta: documenti storici digitalizzati, possibili fondi migrazione e contesto per presenze italiane in Colombia</x:v>
       </x:c>
-      <x:c r="F29" s="10" t="str">
+      <x:c r="F30" s="10" t="str">
         <x:v>Candidato tecnico forte per metadata/discovery: il dataset ufficiale Datos Abiertos Colombia dichiara DataViva come applicazione AGN per consulta, visualizzazione e descarga di piu di 25 milioni di immagini, con accesso OData/Socrata e dati aggiornati nel 2026. Tuttavia i termini generali AGN sono restrittivi su riproduzione/copia/distribuzione dei contenuti; distinguere metadati open data da immagini/documenti e verificare per item prima di qualunque download</x:v>
       </x:c>
-      <x:c r="G29" s="10" t="str">
+      <x:c r="G30" s="10" t="str">
         <x:v>B - forte per futura integrazione metadata/API; download immagini/PDF solo con policy specifica, range esplicito e fixture stabile</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="132" hidden="0" customHeight="1">
-      <x:c r="A30" s="10" t="str">
+    <x:row r="31" ht="158.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A31" s="10" t="str">
         <x:v>nara_catalog</x:v>
       </x:c>
-      <x:c r="B30" s="10" t="str">
+      <x:c r="B31" s="10" t="str">
         <x:v>National Archives Catalog / NARA API</x:v>
       </x:c>
-      <x:c r="C30" s="10" t="str">
+      <x:c r="C31" s="10" t="str">
         <x:v>Stati Uniti / diaspora italiana</x:v>
       </x:c>
-      <x:c r="D30" s="10" t="str">
+      <x:c r="D31" s="10" t="str">
         <x:v>https://www.archives.gov/research/catalog/help/api; https://www.archives.gov/research/immigration/overview</x:v>
       </x:c>
-      <x:c r="E30" s="10" t="str">
+      <x:c r="E31" s="10" t="str">
         <x:v>Alta: naturalizzazioni, immigrazione, passenger records, A-files</x:v>
       </x:c>
-      <x:c r="F30" s="10" t="str">
+      <x:c r="F31" s="10" t="str">
         <x:v>API ufficiale per dati pubblici del Catalog; disponibilita immagini e diritti variano per record</x:v>
       </x:c>
-      <x:c r="G30" s="10" t="str">
+      <x:c r="G31" s="10" t="str">
         <x:v>A/B - candidato forte per metadata/record pubblici</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="237.60000610351562" hidden="0" customHeight="1">
-      <x:c r="A31" s="10" t="str">
-        <x:v>loc_chronicling_america</x:v>
-      </x:c>
-      <x:c r="B31" s="10" t="str">
-        <x:v>Library of Congress - Chronicling America / loc.gov API</x:v>
-      </x:c>
-      <x:c r="C31" s="10" t="str">
-        <x:v>Stati Uniti / contesto diaspora</x:v>
-      </x:c>
-      <x:c r="D31" s="10" t="str">
-        <x:v>https://www.loc.gov/apis/additional-apis/chronicling-america-api/</x:v>
-      </x:c>
-      <x:c r="E31" s="10" t="str">
-        <x:v>Media: giornali storici utili per contesto familiare, non atti vitali</x:v>
-      </x:c>
-      <x:c r="F31" s="10" t="str">
-        <x:v>API ufficiale; utile come modulo di ricerca contestuale piu che downloader genealogico primario</x:v>
-      </x:c>
-      <x:c r="G31" s="10" t="str">
-        <x:v>B - valutare dopo fonti archivistiche</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A32" s="10" t="str">
+        <x:v>loc_chronicling_america</x:v>
+      </x:c>
+      <x:c r="B32" s="10" t="str">
+        <x:v>Library of Congress - Chronicling America / loc.gov API</x:v>
+      </x:c>
+      <x:c r="C32" s="10" t="str">
+        <x:v>Stati Uniti / contesto diaspora</x:v>
+      </x:c>
+      <x:c r="D32" s="10" t="str">
+        <x:v>https://www.loc.gov/apis/additional-apis/chronicling-america-api/</x:v>
+      </x:c>
+      <x:c r="E32" s="10" t="str">
+        <x:v>Media: giornali storici utili per contesto familiare, non atti vitali</x:v>
+      </x:c>
+      <x:c r="F32" s="10" t="str">
+        <x:v>API ufficiale; utile come modulo di ricerca contestuale piu che downloader genealogico primario</x:v>
+      </x:c>
+      <x:c r="G32" s="10" t="str">
+        <x:v>B - valutare dopo fonti archivistiche</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="132" hidden="0" customHeight="1">
+      <x:c r="A33" s="10" t="str">
         <x:v>naa_recordsearch</x:v>
       </x:c>
-      <x:c r="B32" s="10" t="str">
+      <x:c r="B33" s="10" t="str">
         <x:v>National Archives of Australia - RecordSearch passenger arrivals</x:v>
       </x:c>
-      <x:c r="C32" s="10" t="str">
+      <x:c r="C33" s="10" t="str">
         <x:v>Australia / diaspora italiana</x:v>
       </x:c>
-      <x:c r="D32" s="10" t="str">
+      <x:c r="D33" s="10" t="str">
         <x:v>https://www.naa.gov.au/explore-collection/immigration-and-citizenship/passenger-arrival-records</x:v>
       </x:c>
-      <x:c r="E32" s="10" t="str">
+      <x:c r="E33" s="10" t="str">
         <x:v>Alta: arrivi passeggeri 1898-1972, dati migratori</x:v>
       </x:c>
-      <x:c r="F32" s="10" t="str">
+      <x:c r="F33" s="10" t="str">
         <x:v>Fonte ufficiale e molto rilevante; API non confermata, diritti/download da verificare</x:v>
       </x:c>
-      <x:c r="G32" s="10" t="str">
+      <x:c r="G33" s="10" t="str">
         <x:v>B/C - candidato prioritario, inizialmente link assistito</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="224.39999389648438" hidden="0" customHeight="1">
-      <x:c r="A33" s="10" t="str">
+    <x:row r="34" ht="237.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A34" s="10" t="str">
         <x:v>papers_past_digitalnz</x:v>
       </x:c>
-      <x:c r="B33" s="10" t="str">
+      <x:c r="B34" s="10" t="str">
         <x:v>Papers Past / DigitalNZ API</x:v>
       </x:c>
-      <x:c r="C33" s="10" t="str">
+      <x:c r="C34" s="10" t="str">
         <x:v>Nuova Zelanda / diaspora italiana</x:v>
       </x:c>
-      <x:c r="D33" s="10" t="str">
+      <x:c r="D34" s="10" t="str">
         <x:v>https://natlib.govt.nz/about-us/open-data/papers-past-metadata/papers-past-data-using-the-digitalnz-api; https://paperspast.natlib.govt.nz/help/using-papers-past-material</x:v>
       </x:c>
-      <x:c r="E33" s="10" t="str">
+      <x:c r="E34" s="10" t="str">
         <x:v>Media: giornali e avvisi utili per tracce migratorie e familiari</x:v>
       </x:c>
-      <x:c r="F33" s="10" t="str">
+      <x:c r="F34" s="10" t="str">
         <x:v>API metadata ufficiale via DigitalNZ; immagini/testi e copyright da verificare per item</x:v>
       </x:c>
-      <x:c r="G33" s="10" t="str">
+      <x:c r="G34" s="10" t="str">
         <x:v>B - candidato per ricerca contestuale</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="198" hidden="0" customHeight="1">
-      <x:c r="A34" s="10" t="str">
+    <x:row r="35" ht="158.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A35" s="10" t="str">
         <x:v>francearchives</x:v>
       </x:c>
-      <x:c r="B34" s="10" t="str">
+      <x:c r="B35" s="10" t="str">
         <x:v>FranceArchives open data</x:v>
       </x:c>
-      <x:c r="C34" s="10" t="str">
+      <x:c r="C35" s="10" t="str">
         <x:v>Francia / diaspora italiana</x:v>
       </x:c>
-      <x:c r="D34" s="10" t="str">
+      <x:c r="D35" s="10" t="str">
         <x:v>https://francearchives.gouv.fr/fr/open_data</x:v>
       </x:c>
-      <x:c r="E34" s="10" t="str">
+      <x:c r="E35" s="10" t="str">
         <x:v>Alta per ricerche in Francia e migrazioni confinanti</x:v>
       </x:c>
-      <x:c r="F34" s="10" t="str">
+      <x:c r="F35" s="10" t="str">
         <x:v>Dati aperti e aggregazione di inventari; immagini e archivi dipartimentali dipendono dai provider</x:v>
       </x:c>
-      <x:c r="G34" s="10" t="str">
+      <x:c r="G35" s="10" t="str">
         <x:v>B - ottimo per discovery, download solo per provider verificati</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="211.1999969482422" hidden="0" customHeight="1">
-      <x:c r="A35" s="10" t="str">
+    <x:row r="36" ht="224.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A36" s="10" t="str">
         <x:v>belgium_state_archives</x:v>
       </x:c>
-      <x:c r="B35" s="10" t="str">
+      <x:c r="B36" s="10" t="str">
         <x:v>State Archives of Belgium / AGATHA</x:v>
       </x:c>
-      <x:c r="C35" s="10" t="str">
+      <x:c r="C36" s="10" t="str">
         <x:v>Belgio / diaspora italiana</x:v>
       </x:c>
-      <x:c r="D35" s="10" t="str">
+      <x:c r="D36" s="10" t="str">
         <x:v>https://archives.brussels.be/genealogy; https://news.belgium.be/fr/registres-paroissiaux-et-de-letat-civil-consultables-en-ligne-gratuitement</x:v>
       </x:c>
-      <x:c r="E35" s="10" t="str">
+      <x:c r="E36" s="10" t="str">
         <x:v>Alta: stato civile e registri parrocchiali</x:v>
       </x:c>
-      <x:c r="F35" s="10" t="str">
+      <x:c r="F36" s="10" t="str">
         <x:v>Consultazione gratuita ma storicamente richiede account/login per archivi online; non automatizzare accessi autenticati</x:v>
       </x:c>
-      <x:c r="G35" s="10" t="str">
+      <x:c r="G36" s="10" t="str">
         <x:v>C - link/manuale, no integrazione diretta se login necessario</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="264" hidden="0" customHeight="1">
-      <x:c r="A36" s="10" t="str">
+    <x:row r="37" ht="198" hidden="0" customHeight="1">
+      <x:c r="A37" s="10" t="str">
         <x:v>deutsche_digitale_bibliothek</x:v>
       </x:c>
-      <x:c r="B36" s="10" t="str">
+      <x:c r="B37" s="10" t="str">
         <x:v>Deutsche Digitale Bibliothek / DDB API</x:v>
       </x:c>
-      <x:c r="C36" s="10" t="str">
+      <x:c r="C37" s="10" t="str">
         <x:v>Germania / diaspora italiana</x:v>
       </x:c>
-      <x:c r="D36" s="10" t="str">
+      <x:c r="D37" s="10" t="str">
         <x:v>https://www.deutsche-digitale-bibliothek.de/content/api-nutzungsbedingungen?lang=en; https://labs.deutsche-digitale-bibliothek.de/app/ddbapi/</x:v>
       </x:c>
-      <x:c r="E36" s="10" t="str">
+      <x:c r="E37" s="10" t="str">
         <x:v>Media-alta: aggregatore culturale/archivistico tedesco</x:v>
       </x:c>
-      <x:c r="F36" s="10" t="str">
+      <x:c r="F37" s="10" t="str">
         <x:v>API ufficiale ma richiede API key; diritti e contenuti digitali dipendono dai provider</x:v>
       </x:c>
-      <x:c r="G36" s="10" t="str">
+      <x:c r="G37" s="10" t="str">
         <x:v>B/C - metadata possibile, immagini solo item-by-item</x:v>
       </x:c>
     </x:row>
-    <x:row r="37">
-      <x:c r="A37" t="str">
+    <x:row r="38" ht="211.1999969482422" hidden="0" customHeight="1">
+      <x:c r="A38" s="10" t="str">
         <x:v>austrian_state_archives_ais</x:v>
       </x:c>
-      <x:c r="B37" t="str">
+      <x:c r="B38" s="10" t="str">
         <x:v>Oesterreichisches Staatsarchiv - AIS</x:v>
       </x:c>
-      <x:c r="C37" t="str">
+      <x:c r="C38" s="10" t="str">
         <x:v>Austria / area asburgica</x:v>
       </x:c>
-      <x:c r="D37" t="str">
+      <x:c r="D38" s="10" t="str">
         <x:v>https://www.oesta.gv.at/benutzung/Recherche-zu-Hause/recherche/bestande-ais.html; https://www.statearchives.gv.at/user-information/holdings.html</x:v>
       </x:c>
-      <x:c r="E37" t="str">
+      <x:c r="E38" s="10" t="str">
         <x:v>Alta per Lombardo-Veneto, Trentino-Alto Adige, Friuli Venezia Giulia e fonti militari/asburgiche</x:v>
       </x:c>
-      <x:c r="F37" t="str">
+      <x:c r="F38" s="10" t="str">
         <x:v>Sistema ufficiale di ricerca; utile per discovery e ordinazioni, non ancora candidato downloader</x:v>
       </x:c>
-      <x:c r="G37" t="str">
+      <x:c r="G38" s="10" t="str">
         <x:v>C - link/discovery assistito</x:v>
       </x:c>
     </x:row>
-    <x:row r="38">
-      <x:c r="A38" t="str">
+    <x:row r="39" ht="264" hidden="0" customHeight="1">
+      <x:c r="A39" s="10" t="str">
         <x:v>anno_onb</x:v>
       </x:c>
-      <x:c r="B38" t="str">
+      <x:c r="B39" s="10" t="str">
         <x:v>ANNO - AustriaN Newspapers Online</x:v>
       </x:c>
-      <x:c r="C38" t="str">
+      <x:c r="C39" s="10" t="str">
         <x:v>Austria / area asburgica</x:v>
       </x:c>
-      <x:c r="D38" t="str">
+      <x:c r="D39" s="10" t="str">
         <x:v>https://dbis.ur.de/detail.php?bib_id=FUH&amp;lang=en&amp;titel_id=2012; https://www.bundeskanzleramt.gv.at/en/services/federal-administrative-library/databases/general-access-databases.html</x:v>
       </x:c>
-      <x:c r="E38" t="str">
+      <x:c r="E39" s="10" t="str">
         <x:v>Media: giornali storici per contesto migratorio, militare e civile</x:v>
       </x:c>
-      <x:c r="F38" t="str">
+      <x:c r="F39" s="10" t="str">
         <x:v>Fonte pubblica importante; API ufficiale non confermata nel primo passaggio, evitare scraping massivo</x:v>
       </x:c>
-      <x:c r="G38" t="str">
+      <x:c r="G39" s="10" t="str">
         <x:v>C/B - rivalutare se emerge API stabile o download consentito</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Prepare ATK-Pro v3.0.1 RC1 (#376)
</commit_message>
<xml_diff>
--- a/docs_generali/Matrice_portali.xlsx
+++ b/docs_generali/Matrice_portali.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrice portali esistenti" sheetId="1" r:id="R74293ec425ac473e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrice portali candidati" sheetId="2" r:id="R70264843059648eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrice portali esistenti" sheetId="1" r:id="Rf4a02dee58de47a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrice portali candidati" sheetId="2" r:id="Re954a49c67f74d55"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -469,7 +469,7 @@
         <x:v>Supportare solo risorse pubbliche/no-login e verificare condizioni del singolo ente</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="132" hidden="0" customHeight="1">
+    <x:row r="8" ht="211.1999969482422" hidden="0" customHeight="1">
       <x:c r="A8" s="10" t="str">
         <x:v>biblioteca_digitale_siena</x:v>
       </x:c>
@@ -492,7 +492,7 @@
         <x:v>Supportare solo manifest item-level pubblici BDS, con range esplicito, ritmo prudente e verifica delle condizioni del singolo oggetto</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="198" hidden="0" customHeight="1">
+    <x:row r="9" ht="132" hidden="0" customHeight="1">
       <x:c r="A9" s="10" t="str">
         <x:v>bub_digitale</x:v>
       </x:c>
@@ -561,7 +561,7 @@
         <x:v>Supportare solo manifest item-level pubblici, evitare collection di annata, usare range esplicito e controllo diritti/licenza del record</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="224.39999389648438" hidden="0" customHeight="1">
+    <x:row r="12" ht="184.8000030517578" hidden="0" customHeight="1">
       <x:c r="A12" s="10" t="str">
         <x:v>phaidra_unipd</x:v>
       </x:c>
@@ -584,7 +584,7 @@
         <x:v>Supportare solo manifest item-level pubblici, con range esplicito e verifica obbligatoria di rights notice/licenza del singolo oggetto</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="211.1999969482422" hidden="0" customHeight="1">
+    <x:row r="13" ht="198" hidden="0" customHeight="1">
       <x:c r="A13" s="10" t="str">
         <x:v>biblioteca_digitale_trentina</x:v>
       </x:c>
@@ -607,7 +607,7 @@
         <x:v>Supporto tecnico su immagini pubbliche; quando l'utente richiede solo PDF e non imposta range, usare il PDF diretto ufficiale</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="145.1999969482422" hidden="0" customHeight="1">
+    <x:row r="14" ht="224.39999389648438" hidden="0" customHeight="1">
       <x:c r="A14" s="10" t="str">
         <x:v>biblioteca_digitale_lombarda</x:v>
       </x:c>
@@ -630,7 +630,7 @@
         <x:v>Supportare solo documento singolo PDF da endpoint REST pubblico; niente immagini, registro o sequenze finche IIIF/info.json non risultano stabili</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="145.1999969482422" hidden="0" customHeight="1">
+    <x:row r="15" ht="211.1999969482422" hidden="0" customHeight="1">
       <x:c r="A15" s="10" t="str">
         <x:v>rovereto_digital_library</x:v>
       </x:c>
@@ -653,7 +653,7 @@
         <x:v>Supportare solo bitstream classificati come pagine iiifpdf-*.png, con range esplicito per record e controllo licenza del singolo item</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="145.1999969482422" hidden="0" customHeight="1">
+    <x:row r="16" ht="264" hidden="0" customHeight="1">
       <x:c r="A16" s="10" t="str">
         <x:v>doge_unige</x:v>
       </x:c>
@@ -676,7 +676,7 @@
         <x:v>Supportare solo derivati pubblici IIIF-ALTERNATIVE-LD e PDF IIIF-ALTERNATIVE-DOWNLOAD, con range esplicito; escludere ORIGINAL e bundle IIIF-PDF-* segnati nodownload</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="132" hidden="0" customHeight="1">
+    <x:row r="17" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A17" s="10" t="str">
         <x:v>memooria</x:v>
       </x:c>
@@ -699,7 +699,7 @@
         <x:v>Usare come capability tecnica, non come portale unico: richiedere verifica per ogni istanza</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="171.60000610351562" hidden="0" customHeight="1">
+    <x:row r="18" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A18" s="10" t="str">
         <x:v>vatlib</x:v>
       </x:c>
@@ -722,7 +722,7 @@
         <x:v>Mantenere con avviso forte e senza presentarlo come fonte liberamente riusabile</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="118.80000305175781" hidden="0" customHeight="1">
+    <x:row r="19" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A19" s="10" t="str">
         <x:v>findbuch</x:v>
       </x:c>
@@ -745,7 +745,7 @@
         <x:v>Mantenere solo per risorse pubbliche e range puntuale; non estendere senza termini dell'ente</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="158.39999389648438" hidden="0" customHeight="1">
+    <x:row r="20" ht="132" hidden="0" customHeight="1">
       <x:c r="A20" s="10" t="str">
         <x:v>matricula</x:v>
       </x:c>
@@ -768,7 +768,7 @@
         <x:v>Mantenere con limite non commerciale, no derivati, citazione/link e senza bulk scraping</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="132" hidden="0" customHeight="1">
+    <x:row r="21" ht="171.60000610351562" hidden="0" customHeight="1">
       <x:c r="A21" s="10" t="str">
         <x:v>gallica</x:v>
       </x:c>
@@ -791,7 +791,7 @@
         <x:v>Consolidare con citazione obbligatoria, rispetto del non commerciale e cautela sui partner</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="158.39999389648438" hidden="0" customHeight="1">
+    <x:row r="22" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A22" s="10" t="str">
         <x:v>heidelberg</x:v>
       </x:c>
@@ -814,7 +814,7 @@
         <x:v>Consolidare con credito fonte e controllo licenza per singolo volume</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="145.1999969482422" hidden="0" customHeight="1">
+    <x:row r="23" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A23" s="10" t="str">
         <x:v>bodleian</x:v>
       </x:c>
@@ -837,7 +837,7 @@
         <x:v>Consolidare IIIF con avviso non commerciale, attribuzione e niente re-hosting sistematico immagini</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="171.60000610351562" hidden="0" customHeight="1">
+    <x:row r="24" ht="132" hidden="0" customHeight="1">
       <x:c r="A24" s="10" t="str">
         <x:v>e_rara</x:v>
       </x:c>
@@ -860,7 +860,7 @@
         <x:v>Consolidare con controllo licenza per documento e citazione della fonte</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="132" hidden="0" customHeight="1">
+    <x:row r="25" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A25" s="10" t="str">
         <x:v>e_codices</x:v>
       </x:c>
@@ -883,7 +883,7 @@
         <x:v>Consolidare con citazione obbligatoria e avviso per usi commerciali/pubblicazioni</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="79.19999694824219" hidden="0" customHeight="1">
+    <x:row r="26" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A26" s="10" t="str">
         <x:v>e_manuscripta</x:v>
       </x:c>
@@ -906,72 +906,72 @@
         <x:v>Consolidare con controllo licenza per documento; evitare copia sistematica/re-hosting</x:v>
       </x:c>
     </x:row>
-    <x:row r="27">
-      <x:c r="A27" t="str">
+    <x:row r="27" ht="171.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A27" s="10" t="str">
         <x:v>internet_archive</x:v>
       </x:c>
-      <x:c r="B27" t="str">
+      <x:c r="B27" s="10" t="str">
         <x:v>Internet Archive</x:v>
       </x:c>
-      <x:c r="C27" t="str">
+      <x:c r="C27" s="10" t="str">
         <x:v>Internazionale</x:v>
       </x:c>
-      <x:c r="D27" t="str">
+      <x:c r="D27" s="10" t="str">
         <x:v>Manifest sintetico da metadata/files/BookReaderImages</x:v>
       </x:c>
-      <x:c r="E27" t="str">
+      <x:c r="E27" s="10" t="str">
         <x:v>Medio-Alto</x:v>
       </x:c>
-      <x:c r="F27" t="str">
+      <x:c r="F27" s="10" t="str">
         <x:v>Licenza e disponibilita variabili per item; alcuni item sono prestito o no-download</x:v>
       </x:c>
-      <x:c r="G27" t="str">
+      <x:c r="G27" s="10" t="str">
         <x:v>Supportare solo item pubblici scaricabili, con licenza/diritti chiari e senza aggirare prestito/no-download</x:v>
       </x:c>
     </x:row>
-    <x:row r="28">
-      <x:c r="A28" t="str">
+    <x:row r="28" ht="132" hidden="0" customHeight="1">
+      <x:c r="A28" s="10" t="str">
         <x:v>europeana</x:v>
       </x:c>
-      <x:c r="B28" t="str">
+      <x:c r="B28" s="10" t="str">
         <x:v>Europeana IIIF</x:v>
       </x:c>
-      <x:c r="C28" t="str">
+      <x:c r="C28" s="10" t="str">
         <x:v>Internazionale</x:v>
       </x:c>
-      <x:c r="D28" t="str">
+      <x:c r="D28" s="10" t="str">
         <x:v>IIIF diretto da provider/record id</x:v>
       </x:c>
-      <x:c r="E28" t="str">
+      <x:c r="E28" s="10" t="str">
         <x:v>Basso-Medio</x:v>
       </x:c>
-      <x:c r="F28" t="str">
+      <x:c r="F28" s="10" t="str">
         <x:v>Diritti da leggere per record/provider; API soggetta a chiave, termini e limiti</x:v>
       </x:c>
-      <x:c r="G28" t="str">
+      <x:c r="G28" s="10" t="str">
         <x:v>Usare solo record con IIIF disponibile, rights statement chiaro e attribution ai provider</x:v>
       </x:c>
     </x:row>
-    <x:row r="29">
-      <x:c r="A29" t="str">
+    <x:row r="29" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A29" s="10" t="str">
         <x:v>manifest_diretto</x:v>
       </x:c>
-      <x:c r="B29" t="str">
+      <x:c r="B29" s="10" t="str">
         <x:v>Manifest diretto (URL gia noto)</x:v>
       </x:c>
-      <x:c r="C29" t="str">
+      <x:c r="C29" s="10" t="str">
         <x:v>Avanzato</x:v>
       </x:c>
-      <x:c r="D29" t="str">
+      <x:c r="D29" s="10" t="str">
         <x:v>URL manifest fornito dall'utente</x:v>
       </x:c>
-      <x:c r="E29" t="str">
+      <x:c r="E29" s="10" t="str">
         <x:v>Variabile</x:v>
       </x:c>
-      <x:c r="F29" t="str">
+      <x:c r="F29" s="10" t="str">
         <x:v>Responsabilita utente + verifica termini origine</x:v>
       </x:c>
-      <x:c r="G29" t="str">
+      <x:c r="G29" s="10" t="str">
         <x:v>Mantenere con avviso/criteri chiari</x:v>
       </x:c>
     </x:row>
@@ -1016,7 +1016,7 @@
         <x:v>Decisione provvisoria</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="382.79998779296875" hidden="0" customHeight="1">
+    <x:row r="2" ht="976.7999877929688" hidden="0" customHeight="1">
       <x:c r="A2" s="10" t="str">
         <x:v>archivi_nazionali</x:v>
       </x:c>
@@ -1039,7 +1039,7 @@
         <x:v>C - candidato strategico per discovery/link assistito e accesso ai servizi; nessun downloader finche non emergono API/IIIF/endpoint pubblici compatibili</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="488.3999938964844" hidden="0" customHeight="1">
+    <x:row r="3" ht="765.5999755859375" hidden="0" customHeight="1">
       <x:c r="A3" s="10" t="str">
         <x:v>archivio_digitale_icar</x:v>
       </x:c>
@@ -1062,7 +1062,7 @@
         <x:v>C - link/discovery assistito e consultazione pubblica; vietare builder/downloader e live smoke di download salvo futuro endpoint ufficiale documentato e autorizzato</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="528" hidden="0" customHeight="1">
+    <x:row r="4" ht="673.2000122070312" hidden="0" customHeight="1">
       <x:c r="A4" s="10" t="str">
         <x:v>sias</x:v>
       </x:c>
@@ -1085,7 +1085,7 @@
         <x:v>C - discovery/link assistito e apertura inventari; no download immagini o PDF massivo senza endpoint e termini specifici</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="475.20001220703125" hidden="0" customHeight="1">
+    <x:row r="5" ht="871.2000122070312" hidden="0" customHeight="1">
       <x:c r="A5" s="10" t="str">
         <x:v>san_risorse_digitali</x:v>
       </x:c>
@@ -1108,7 +1108,7 @@
         <x:v>B - capability futura metadata/OAI piu' concreta; no downloader immagini diretto via SAN</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="462" hidden="0" customHeight="1">
+    <x:row r="6" ht="633.5999755859375" hidden="0" customHeight="1">
       <x:c r="A6" s="10" t="str">
         <x:v>siusa</x:v>
       </x:c>
@@ -1131,7 +1131,7 @@
         <x:v>C - discovery, schede e link assistito; eventuale metadata solo via SAN/open data, nessun downloader</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="660" hidden="0" customHeight="1">
+    <x:row r="7" ht="1016.4000244140625" hidden="0" customHeight="1">
       <x:c r="A7" s="10" t="str">
         <x:v>beweb</x:v>
       </x:c>
@@ -1154,7 +1154,7 @@
         <x:v>C - discovery/link assistito e, al massimo, futura metadata/search su dati catalografici compatibili; no downloader generico</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="541.2000122070312" hidden="0" customHeight="1">
+    <x:row r="8" ht="1016.4000244140625" hidden="0" customHeight="1">
       <x:c r="A8" s="10" t="str">
         <x:v>archivi_diocesani_italiani</x:v>
       </x:c>
@@ -1177,9 +1177,9 @@
         <x:v>C - mappa/link assistiti e schede di orientamento; vietare automazioni generiche, login, aree riservate e download senza fonte pubblica no-login con termini chiari</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="712.7999877929688" hidden="0" customHeight="1">
+    <x:row r="9" ht="607.2000122070312" hidden="0" customHeight="1">
       <x:c r="A9" s="10" t="str">
-        <x:v>archivio_stato_ticino / servizio_archivi_locali_ticino</x:v>
+        <x:v>asti_scopearchiv / asti_mappe_catastali / asti_fondi_fotografici / asti_pergamene</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
         <x:v>Archivio di Stato del Cantone Ticino / SAL</x:v>
@@ -1188,19 +1188,19 @@
         <x:v>Svizzera italiana</x:v>
       </x:c>
       <x:c r="D9" s="10" t="str">
-        <x:v>https://www4.ti.ch/decs/dcsu/asti/servizi/servizio-archivi-locali-sal/; https://www4.ti.ch/fileadmin/DECS/DCSU/ASTI/Documenti/Ricerche_genealogiche.pdf; https://www4.ti.ch/decs/dcsu/asti/servizi/consultazione-e-riproduzione-dei-documenti/; catalogo https://www.archiviodistato.ti.ch/Query/volltextsuche.aspx</x:v>
+        <x:v>https://www4.ti.ch/decs/dcsu/asti/; catalogo https://www.archiviodistato.ti.ch/Query/volltextsuche.aspx; nota tecnica candidati_svizzeri_prossima_release_SAG_ASTi.md</x:v>
       </x:c>
       <x:c r="E9" s="10" t="str">
-        <x:v>Molto alta per Ticino: fondi genealogici 1750-1960, archivi comunali, patriziali e parrocchiali, ruoli di popolazione, stato civile e microfilm ecclesiastici</x:v>
+        <x:v>Molto alta per Ticino: fondi genealogici, archivi comunali e parrocchiali, mappe catastali, fotografie e pergamene</x:v>
       </x:c>
       <x:c r="F9" s="10" t="str">
-        <x:v>Controllo 2026-06-05 + ricontrollo ufficiale 2026-07-31: ASTi/SAL continua a censire e riordinare archivi locali, compresi archivi parrocchiali, e offre strumenti online reali come il catalogo scopeArchiv. La consultazione in sede o in versione digitale resta gratuita, ma regolamento e tariffario confermano emolumenti per alcuni servizi, comprese riproduzioni digitali e supporti di ricerca approfonditi. Le ricerche genealogiche restano soggette a condizioni particolari e a richieste puntuali via formulario; i registri parrocchiali ticinesi risultano ancora accessibili soprattutto tramite FamilySearch o microfilm presso l'Archivio diocesano di Lugano, non come endpoint pubblico ASTi</x:v>
+        <x:v>Verifica 2026-09-27: il perimetro non e' omogeneo. scopeArchiv e pergamene sono soprattutto discovery; le mappe catastali espongono immagini Zoomify recuperabili con selezione esplicita; i fondi fotografici richiedono ancora sonda endpoint e verifica diritti. Ruoli, stato civile e registri parrocchiali restano soggetti a condizioni particolari e non costituiscono un corpus pubblico scaricabile</x:v>
       </x:c>
       <x:c r="G9" s="10" t="str">
-        <x:v>C - link/manuale e schede di orientamento; no downloader ATK-Pro</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="369.6000061035156" hidden="0" customHeight="1">
+        <x:v>B per asti_mappe_catastali con R_LIMITED; REVIEW per fotografie; C discovery per scopeArchiv e pergamene</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="712.7999877929688" hidden="0" customHeight="1">
       <x:c r="A10" s="10" t="str">
         <x:v>archivio_diocesano_lugano</x:v>
       </x:c>
@@ -1223,647 +1223,670 @@
         <x:v>C - solo contatto/link assistito e istruzioni di consultazione</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="686.4000244140625" hidden="0" customHeight="1">
+    <x:row r="11" ht="501.6000061035156" hidden="0" customHeight="1">
       <x:c r="A11" s="10" t="str">
-        <x:v>archivio_stato_grigioni</x:v>
+        <x:v>sag_cmi_ais</x:v>
       </x:c>
       <x:c r="B11" s="10" t="str">
-        <x:v>Archivio di Stato dei Grigioni</x:v>
+        <x:v>Archivio di Stato dei Grigioni (SAG)</x:v>
       </x:c>
       <x:c r="C11" s="10" t="str">
         <x:v>Grigioni italofoni / area retica</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
-        <x:v>https://www.gr.ch/IT/istituzioni/amministrazione/ekud/afk/sag/servizi/fondi/familienforschung/Seiten/default.aspx; https://www.gr.ch/IT/istituzioni/amministrazione/ekud/afk/sag/servizi/fondi/Seiten/default.aspx; https://www.gr.ch/IT/istituzioni/amministrazione/ekud/afk/sag/chisiamo/Seiten/default.aspx</x:v>
+        <x:v>catalogo CMI AIS e nota tecnica candidati_svizzeri_prossima_release_SAG_ASTi.md; https://www.gr.ch/IT/istituzioni/amministrazione/ekud/afk/sag/</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
-        <x:v>Molto alta per valli italofone, mobilita alpina e fonti pre-1876: registri parrocchiali, stato civile, registri dei cittadini, schede genealogiche e strumenti di ricerca</x:v>
+        <x:v>Molto alta per valli italofone, mobilita alpina e fonti pre-1876: registri parrocchiali, stato civile, registri dei cittadini e microfilm</x:v>
       </x:c>
       <x:c r="F11" s="10" t="str">
-        <x:v>Controllo 2026-06-05 + ricontrollo ufficiale 2026-07-31: l'Archivio di Stato conferma che tutti i registri parrocchiali noti sono stati microfilmati e consultabili presso l'Archivio; i registri di stato civile fino al 1929 sono consultabili in sala di lettura, quelli dei cittadini attinenti fino al 1929 su microfilm, mentre i registri delle famiglie dal 1929 non sono visionabili. Il quadro online e' piu' ricco di quanto sembrasse: oltre a PDF e sistema informativo, il sito indica fondi digitalizzati consultabili online e integrazione con Archives Online per metadati e documenti delle banche dati collegate. Resta comunque un ramo soprattutto consultativo e regolato</x:v>
+        <x:v>Verifica pratica 2026-09-27: le API pubbliche CMI AIS consentono ricerca e dettaglio; per numerosi record liberamente accessibili e' disponibile il PDF originale senza login. L'adapter deve rispettare lo stato di accesso item-level, usare streaming, limiti e nomi sicuri e non estendere il download ai record protetti</x:v>
       </x:c>
       <x:c r="G11" s="10" t="str">
-        <x:v>C - discovery/link assistito; no download generale, salvo eventuali fondi digitalizzati con condizioni specifiche</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="435.6000061035156" hidden="0" customHeight="1">
+        <x:v>A - adapter sag_cmi_ais, politica iniziale D_ONLY, priorita' della prossima release funzionale</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="712.7999877929688" hidden="0" customHeight="1">
       <x:c r="A12" s="10" t="str">
+        <x:v>biblioteca_cremona_filestation</x:v>
+      </x:c>
+      <x:c r="B12" s="10" t="str">
+        <x:v>Biblioteca Statale di Cremona - raccolte digitali File Station</x:v>
+      </x:c>
+      <x:c r="C12" s="10" t="str">
+        <x:v>Lombardia / stampa e raccolte locali</x:v>
+      </x:c>
+      <x:c r="D12" s="10" t="str">
+        <x:v>https://bibliocremona.it/patrimonio/biblioteca-digitale/risorse-elettroniche/la-provincia-1883-1923/; https://bibliocremona.it/patrimonio/biblioteca-digitale/; nota tecnica prossima_release_AI_e_Biblioteca_Cremona.md</x:v>
+      </x:c>
+      <x:c r="E12" s="10" t="str">
+        <x:v>Alta: quotidiani storici, materiali digitalizzati e risorse accessibili, con JPEG, PDF e XML strutturato</x:v>
+      </x:c>
+      <x:c r="F12" s="10" t="str">
+        <x:v>Verifica pratica 2026-09-27: API Synology File Station e quattro condivisioni leggibili (LA PROVINCIA, IL REGIME FASCISTA, MATERIALE DIGITALIZZATO, LIS). Un solo connettore puo' esporre quattro profili; le altre risorse del sito richiedono analisi separate. Bloccanti: endpoint IP con certificato non valido per il nome host, credenziali pubbliche soggette a rotazione e condizioni di automazione, attribuzione e riuso non ancora esplicite</x:v>
+      </x:c>
+      <x:c r="G12" s="10" t="str">
+        <x:v>B / HOLD - famiglia synology_file_station, politica proposta R_LIMITED; implementare solo dopo TLS valido e conferma scritta</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="739.2000122070312" hidden="0" customHeight="1">
+      <x:c r="A13" s="10" t="str">
         <x:v>diocesi_chur_coira</x:v>
       </x:c>
-      <x:c r="B12" s="10" t="str">
+      <x:c r="B13" s="10" t="str">
         <x:v>Archivio vescovile di Coira / Bischöfliches Archiv Chur</x:v>
       </x:c>
-      <x:c r="C12" s="10" t="str">
+      <x:c r="C13" s="10" t="str">
         <x:v>Grigioni / area retica ecclesiastica</x:v>
       </x:c>
-      <x:c r="D12" s="10" t="str">
+      <x:c r="D13" s="10" t="str">
         <x:v>https://www.archiv-bistum-chur.ch/; https://www.bistumsarchiv-chur.findbuch.net/; contatti https://www.archiv-bistum-chur.ch/Kontakt.htm</x:v>
       </x:c>
-      <x:c r="E12" s="10" t="str">
+      <x:c r="E13" s="10" t="str">
         <x:v>Alta: diocesi storica antica, rilevante per fonti ecclesiastiche grigionesi e area retica</x:v>
       </x:c>
-      <x:c r="F12" s="10" t="str">
+      <x:c r="F13" s="10" t="str">
         <x:v>Ricontrollo ufficiale 2026-07-31: il sito documenta un archivio ecclesiastico strutturato, con ordinamento dei fondi, repertori online, Findbuch e lavori di digitalizzazione/descrizione in corso su varie serie. La pagina contatti esplicita pero' che il BAC non e' un archivio pubblico: la consultazione e' solo previa richiesta, nel locale di lettura/lavoro e secondo un regolamento proprio. Non emerge quindi una policy di download immagini/API generalizzabile</x:v>
       </x:c>
-      <x:c r="G12" s="10" t="str">
+      <x:c r="G13" s="10" t="str">
         <x:v>C - link/discovery assistito; non estendere come downloader generico</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="396" hidden="0" customHeight="1">
-      <x:c r="A13" s="10" t="str">
+    <x:row r="14" ht="396" hidden="0" customHeight="1">
+      <x:c r="A14" s="10" t="str">
         <x:v>biblioteca_digitale_siena</x:v>
       </x:c>
-      <x:c r="B13" s="10" t="str">
+      <x:c r="B14" s="10" t="str">
         <x:v>Biblioteca Digitale Siena</x:v>
       </x:c>
-      <x:c r="C13" s="10" t="str">
+      <x:c r="C14" s="10" t="str">
         <x:v>Italia</x:v>
       </x:c>
-      <x:c r="D13" s="10" t="str">
+      <x:c r="D14" s="10" t="str">
         <x:v>https://bds.comune.siena.it/; https://bds.comune.siena.it/it/169/</x:v>
       </x:c>
-      <x:c r="E13" s="10" t="str">
+      <x:c r="E14" s="10" t="str">
         <x:v>Media-alta: manoscritti, periodici, disegni, archivi e carteggi senesi/toscani</x:v>
       </x:c>
-      <x:c r="F13" s="10" t="str">
+      <x:c r="F14" s="10" t="str">
         <x:v>Piattaforma pubblica IIIF; termini ufficiali consentono JPG web-resolution per uso personale, studio e ricerca con citazione, vietando uso commerciale e trasformazioni non autorizzate; smoke live 2026-06-05 passato su manifest da 106 canvas</x:v>
       </x:c>
-      <x:c r="G13" s="10" t="str">
+      <x:c r="G14" s="10" t="str">
         <x:v>A - builder viewer-&gt;manifest aggiunto e verificato live</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="448.79998779296875" hidden="0" customHeight="1">
-      <x:c r="A14" s="10" t="str">
+    <x:row r="15" ht="448.79998779296875" hidden="0" customHeight="1">
+      <x:c r="A15" s="10" t="str">
         <x:v>biblioteca_digitale_trentina</x:v>
       </x:c>
-      <x:c r="B14" s="10" t="str">
+      <x:c r="B15" s="10" t="str">
         <x:v>Biblioteca Digitale Trentina</x:v>
       </x:c>
-      <x:c r="C14" s="10" t="str">
+      <x:c r="C15" s="10" t="str">
         <x:v>Italia / Trentino e area ex asburgica</x:v>
       </x:c>
-      <x:c r="D14" s="10" t="str">
+      <x:c r="D15" s="10" t="str">
         <x:v>https://bdt.bibcom.trento.it/; https://bdt.bibcom.trento.it/Riuso; https://www.comune.trento.it/Servizi/Biblioteca-Digitale-Trentina-BDT</x:v>
       </x:c>
-      <x:c r="E14" s="10" t="str">
+      <x:c r="E15" s="10" t="str">
         <x:v>Alta per storia locale, Trentino, mobilita alpina, cartoline, periodici, carte geografiche, stampe e fonti bibliografiche di contesto</x:v>
       </x:c>
-      <x:c r="F14" s="10" t="str">
+      <x:c r="F15" s="10" t="str">
         <x:v>Controllo 2026-06-06: fonte istituzionale pubblica, accesso libero, download gratuito delle immagini e pagina di riuso molto favorevole: materiali in pubblico dominio, riuso anche commerciale con citazione. La sonda ha trovato immagini dirette e PDF diretto, non manifest IIIF reale</x:v>
       </x:c>
-      <x:c r="G14" s="10" t="str">
+      <x:c r="G15" s="10" t="str">
         <x:v>A - promosso a supporto tecnico: manifest sintetico da immagini pubbliche e PDF diretto ufficiale per testi a stampa quando l'utente richiede solo PDF senza range</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="831.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A15" s="10" t="str">
+    <x:row r="16" ht="1095.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A16" s="10" t="str">
         <x:v>beic_digitale</x:v>
       </x:c>
-      <x:c r="B15" s="10" t="str">
+      <x:c r="B16" s="10" t="str">
         <x:v>BEIC digital library</x:v>
-      </x:c>
-      <x:c r="C15" s="10" t="str">
-        <x:v>Italia / Lombardia</x:v>
-      </x:c>
-      <x:c r="D15" s="10" t="str">
-        <x:v>https://digital.beic.it/; https://digital.beic.it/termini-duso/; https://digital.beic.it/infrastruttura-e-standard/; esempi tecnici Preserver https://preserver.beic.it/delivery/DeliveryManagerServlet?dps_pid=IE7400509</x:v>
-      </x:c>
-      <x:c r="E15" s="10" t="str">
-        <x:v>Alta per libri antichi, manoscritti, periodici, editoria lombarda e fonti bibliografiche utili alla ricerca genealogica e territoriale</x:v>
-      </x:c>
-      <x:c r="F15" s="10" t="str">
-        <x:v>Controllo 2026-06-08 + ricontrollo 2026-07-29: termini ufficiali molto favorevoli per opere in pubblico dominio, immagini scaricabili/riutilizzabili e dati CC0; infrastruttura Rosetta/Alma/Primo VE con OAI-PMH documentato. Lato download non e ancora emerso un endpoint utilizzabile in modo ripetibile: il test live su Preserver IE7400509 continua a mostrare solo viewer e logo del sito, mentre il record Primo alma9925210904741 non espone manifest, PDF o immagini utili alla sonda. Il probe ora separa esplicitamente gli asset grafici di sito dai segnali tecnici riusabili e classifica entrambi i campioni come GO/NO-GO: HOLD. verify_beic_technical_probe.py resta lo strumento di raccolta campioni, ma senza integrazione nel menu</x:v>
-      </x:c>
-      <x:c r="G15" s="10" t="str">
-        <x:v>B/C - candidato forte per metadata e valore culturale, ma downloader sospeso finche non emergono campioni BEIC diretti con endpoint file/manifest stabile e policy item-level</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="660" hidden="0" customHeight="1">
-      <x:c r="A16" s="10" t="str">
-        <x:v>biblioteca_digitale_lombarda</x:v>
-      </x:c>
-      <x:c r="B16" s="10" t="str">
-        <x:v>Biblioteca Digitale Lombarda</x:v>
       </x:c>
       <x:c r="C16" s="10" t="str">
         <x:v>Italia / Lombardia</x:v>
       </x:c>
       <x:c r="D16" s="10" t="str">
+        <x:v>https://digital.beic.it/; https://digital.beic.it/termini-duso/; https://digital.beic.it/infrastruttura-e-standard/; esempi tecnici Preserver https://preserver.beic.it/delivery/DeliveryManagerServlet?dps_pid=IE7400509</x:v>
+      </x:c>
+      <x:c r="E16" s="10" t="str">
+        <x:v>Alta per libri antichi, manoscritti, periodici, editoria lombarda e fonti bibliografiche utili alla ricerca genealogica e territoriale</x:v>
+      </x:c>
+      <x:c r="F16" s="10" t="str">
+        <x:v>Controllo 2026-06-08 + ricontrollo 2026-07-29: termini ufficiali molto favorevoli per opere in pubblico dominio, immagini scaricabili/riutilizzabili e dati CC0; infrastruttura Rosetta/Alma/Primo VE con OAI-PMH documentato. Lato download non e ancora emerso un endpoint utilizzabile in modo ripetibile: il test live su Preserver IE7400509 continua a mostrare solo viewer e logo del sito, mentre il record Primo alma9925210904741 non espone manifest, PDF o immagini utili alla sonda. Il probe ora separa esplicitamente gli asset grafici di sito dai segnali tecnici riusabili e classifica entrambi i campioni come GO/NO-GO: HOLD. verify_beic_technical_probe.py resta lo strumento di raccolta campioni, ma senza integrazione nel menu</x:v>
+      </x:c>
+      <x:c r="G16" s="10" t="str">
+        <x:v>B/C - candidato forte per metadata e valore culturale, ma downloader sospeso finche non emergono campioni BEIC diretti con endpoint file/manifest stabile e policy item-level</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="660" hidden="0" customHeight="1">
+      <x:c r="A17" s="10" t="str">
+        <x:v>biblioteca_digitale_lombarda</x:v>
+      </x:c>
+      <x:c r="B17" s="10" t="str">
+        <x:v>Biblioteca Digitale Lombarda</x:v>
+      </x:c>
+      <x:c r="C17" s="10" t="str">
+        <x:v>Italia / Lombardia</x:v>
+      </x:c>
+      <x:c r="D17" s="10" t="str">
         <x:v>https://www.bdl.servizirl.it/; esempi record pubblici https://www.bdl.servizirl.it/vufind/Record/BDL-OGGETTO-133442; endpoint PDF pubblici https://www.bdl.servizirl.it/bdl/public/rest/srv/item/12404/pdf</x:v>
       </x:c>
-      <x:c r="E16" s="10" t="str">
+      <x:c r="E17" s="10" t="str">
         <x:v>Alta per storia locale lombarda, periodici, monografie, archivi e fondi civici</x:v>
       </x:c>
-      <x:c r="F16" s="10" t="str">
+      <x:c r="F17" s="10" t="str">
         <x:v>Controllo 2026-06-08: portale pubblico VuFind con record e PDF REST pubblici; il campione item/12404/pdf risponde come PDF reale ed e promosso a supporto puntuale D_ONLY. La pagina record espone anche una miniatura Cantaloupe/IIIF (6823693) ma insieme ad asset grafici del sito; l'info.json derivato ha dato timeout nel test live. Molti record dichiarano CC BY-NC-ND, quindi uso studio/ricerca con limiti non commerciale/no-derivati</x:v>
       </x:c>
-      <x:c r="G16" s="10" t="str">
+      <x:c r="G17" s="10" t="str">
         <x:v>A/B - promosso solo per PDF puntuale pubblico; niente supporto immagini/registro finche info.json, sequenze o manifest non risultano stabili</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="976.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A17" s="10" t="str">
+    <x:row r="18" ht="976.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A18" s="10" t="str">
         <x:v>ambrosiana_digitale</x:v>
       </x:c>
-      <x:c r="B17" s="10" t="str">
+      <x:c r="B18" s="10" t="str">
         <x:v>Veneranda Biblioteca Ambrosiana - Digital Library</x:v>
       </x:c>
-      <x:c r="C17" s="10" t="str">
+      <x:c r="C18" s="10" t="str">
         <x:v>Italia / Lombardia ecclesiastica e manoscritti</x:v>
       </x:c>
-      <x:c r="D17" s="10" t="str">
+      <x:c r="D18" s="10" t="str">
         <x:v>https://www.ambrosiana.it/en/discover/masterpieces/the-digital-library/; https://ambrosiana.comperio.it/library-digital/; esempi Comperio https://ambrosiana.comperio.it/opac/detail/view/ambro:catalog:24203; campione pubblico UniCatt/Veneranda https://digitallibrary.unicatt.it/veneranda/data/public/manifests/0b/02/da/82/80/0d/10/a0/0b02da82800d10a0.json</x:v>
       </x:c>
-      <x:c r="E17" s="10" t="str">
+      <x:c r="E18" s="10" t="str">
         <x:v>Alta per manoscritti, codici, fondi storici e fonti culturali collegate a Milano e Lombardia</x:v>
       </x:c>
-      <x:c r="F17" s="10" t="str">
+      <x:c r="F18" s="10" t="str">
         <x:v>Controllo 2026-06-07/2026-07-25: la pagina ufficiale descrive accesso libero e uso dello standard IIIF; fonte accademica conferma Mirador e Cantaloupe. Test live su ambro:catalog:24203: trovati solo record Comperio duplicati/correlati e asset grafico, nessun manifest, info.json, immagine Cantaloupe o viewer utile. Verifica aggiuntiva su piattaforma pubblica UniCatt/Veneranda: manifest IIIF scaricato con codice 200 e 101 canvas. La pista tecnica esiste quindi davvero, ma la UI pubblica segnala No Downloadable; senza termini item-level compatibili o autorizzazione esplicita al download, il ramo resta fuori dal downloader</x:v>
       </x:c>
-      <x:c r="G17" s="10" t="str">
+      <x:c r="G18" s="10" t="str">
         <x:v>B/C - valore alto e IIIF pubblico confermato, ma integrazione sospesa per restrizione No Downloadable e assenza di termini item-level che autorizzino il download</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="858" hidden="0" customHeight="1">
-      <x:c r="A18" s="10" t="str">
+    <x:row r="19" ht="858" hidden="0" customHeight="1">
+      <x:c r="A19" s="10" t="str">
         <x:v>rovereto_digital_library</x:v>
       </x:c>
-      <x:c r="B18" s="10" t="str">
+      <x:c r="B19" s="10" t="str">
         <x:v>Rovereto Digital Library / Biblioteca Tartarotti</x:v>
       </x:c>
-      <x:c r="C18" s="10" t="str">
+      <x:c r="C19" s="10" t="str">
         <x:v>Italia / Trentino</x:v>
       </x:c>
-      <x:c r="D18" s="10" t="str">
+      <x:c r="D19" s="10" t="str">
         <x:v>https://digitallibrary.bibliotecacivica.rovereto.tn.it/; campioni https://digitallibrary.bibliotecacivica.rovereto.tn.it/entities/publication/e4199e9b-c79b-4c3d-b157-be2dcfc0407f, https://digitallibrary.bibliotecacivica.rovereto.tn.it/entities/picture/2cbeaeab-833a-48c2-9b39-29484ed1c681; termini https://digitallibrary.bibliotecacivica.rovereto.tn.it/info/end-user-agreement</x:v>
       </x:c>
-      <x:c r="E18" s="10" t="str">
+      <x:c r="E19" s="10" t="str">
         <x:v>Media-alta per storia locale trentina, fotografie, documenti d'archivio, riviste e contesto familiare</x:v>
       </x:c>
-      <x:c r="F18" s="10" t="str">
+      <x:c r="F19" s="10" t="str">
         <x:v>Controllo 2026-06-08: portale operativo DSpace-GLAM promosso a supporto tecnico prudente. ATK-Pro deriva l'endpoint REST item standard, segue la paginazione HAL/JSON di bundle e bitstream, costruisce un manifest sintetico solo dai bitstream pubblici classificati come pagine iiifpdf-*.png e conserva il PDF originale solo come riferimento seeAlso. Restano esclusi licenza, miniature/cover e derivati testuali/OCR. Termini ufficiali: accesso libero e gratuito ai file digitali in risoluzione web secondo licenze specifiche; alta definizione su richiesta</x:v>
       </x:c>
-      <x:c r="G18" s="10" t="str">
+      <x:c r="G19" s="10" t="str">
         <x:v>A - promosso a supporto tecnico R_LIMITED con range esplicito e controllo licenza item-level</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="937.2000122070312" hidden="0" customHeight="1">
-      <x:c r="A19" s="10" t="str">
+    <x:row r="20" ht="937.2000122070312" hidden="0" customHeight="1">
+      <x:c r="A20" s="10" t="str">
         <x:v>bub_digitale</x:v>
       </x:c>
-      <x:c r="B19" s="10" t="str">
+      <x:c r="B20" s="10" t="str">
         <x:v>BUB Digitale / Biblioteca Universitaria di Bologna</x:v>
-      </x:c>
-      <x:c r="C19" s="10" t="str">
-        <x:v>Italia / Emilia-Romagna</x:v>
-      </x:c>
-      <x:c r="D19" s="10" t="str">
-        <x:v>https://bub.unibo.it/it/bub-digitale; https://bub.unibo.it/it/bub-digitale/bollettini-parrocchiali; campioni Bondanello 1934 e Castenaso 1933</x:v>
-      </x:c>
-      <x:c r="E19" s="10" t="str">
-        <x:v>Media-alta: papiri, manoscritti greci/arabi/ebraici, opere a stampa, periodici storici, bollettini parrocchiali, fotografie e fondi bolognesi utili al contesto storico-familiare</x:v>
-      </x:c>
-      <x:c r="F19" s="10" t="str">
-        <x:v>Controllo 2026-06-08: fonte ufficiale BUB descrive accesso libero e gratuito per studio/ricerca, uso dello standard IIIF e visualizzatore Mirador. La landing page live espone soprattutto pagine del portale e immagini Plone @@images, ora classificate come plone_page_image per non confonderle con pagine documento. Test live mirato sul bollettino Bondanello 1934: manifest IIIF v2 pulito da viewer_manifest_parameter, codice 200, 44 canvas. Secondo campione Castenaso 1933: manifest diretto, codice 200, 32 canvas. Pattern manifest stabile su piu bollettini; promosso a supporto IIIF diretto prudente</x:v>
-      </x:c>
-      <x:c r="G19" s="10" t="str">
-        <x:v>A - promosso a supporto R_LIMITED: solo manifest BUB pubblici, range esplicito, referer BUB e verifica licenza item-level</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="871.2000122070312" hidden="0" customHeight="1">
-      <x:c r="A20" s="10" t="str">
-        <x:v>dl_ficlit</x:v>
-      </x:c>
-      <x:c r="B20" s="10" t="str">
-        <x:v>FICLIT Digital Library / Universita di Bologna</x:v>
       </x:c>
       <x:c r="C20" s="10" t="str">
         <x:v>Italia / Emilia-Romagna</x:v>
       </x:c>
       <x:c r="D20" s="10" t="str">
+        <x:v>https://bub.unibo.it/it/bub-digitale; https://bub.unibo.it/it/bub-digitale/bollettini-parrocchiali; campioni Bondanello 1934 e Castenaso 1933</x:v>
+      </x:c>
+      <x:c r="E20" s="10" t="str">
+        <x:v>Media-alta: papiri, manoscritti greci/arabi/ebraici, opere a stampa, periodici storici, bollettini parrocchiali, fotografie e fondi bolognesi utili al contesto storico-familiare</x:v>
+      </x:c>
+      <x:c r="F20" s="10" t="str">
+        <x:v>Controllo 2026-06-08: fonte ufficiale BUB descrive accesso libero e gratuito per studio/ricerca, uso dello standard IIIF e visualizzatore Mirador. La landing page live espone soprattutto pagine del portale e immagini Plone @@images, ora classificate come plone_page_image per non confonderle con pagine documento. Test live mirato sul bollettino Bondanello 1934: manifest IIIF v2 pulito da viewer_manifest_parameter, codice 200, 44 canvas. Secondo campione Castenaso 1933: manifest diretto, codice 200, 32 canvas. Pattern manifest stabile su piu bollettini; promosso a supporto IIIF diretto prudente</x:v>
+      </x:c>
+      <x:c r="G20" s="10" t="str">
+        <x:v>A - promosso a supporto R_LIMITED: solo manifest BUB pubblici, range esplicito, referer BUB e verifica licenza item-level</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="871.2000122070312" hidden="0" customHeight="1">
+      <x:c r="A21" s="10" t="str">
+        <x:v>dl_ficlit</x:v>
+      </x:c>
+      <x:c r="B21" s="10" t="str">
+        <x:v>FICLIT Digital Library / Universita di Bologna</x:v>
+      </x:c>
+      <x:c r="C21" s="10" t="str">
+        <x:v>Italia / Emilia-Romagna</x:v>
+      </x:c>
+      <x:c r="D21" s="10" t="str">
         <x:v>https://dl.ficlit.unibo.it/s/lib/page/progetto; campioni https://dl.ficlit.unibo.it/s/lib/item/199245, https://dl.ficlit.unibo.it/s/lib/item/28429</x:v>
       </x:c>
-      <x:c r="E20" s="10" t="str">
+      <x:c r="E21" s="10" t="str">
         <x:v>Media: collezioni accademiche e umanistiche, fonti letterarie, bibliografiche e documentarie utili a ricerche storiche territoriali</x:v>
       </x:c>
-      <x:c r="F20" s="10" t="str">
+      <x:c r="F21" s="10" t="str">
         <x:v>Controllo 2026-06-08: fonte ufficiale descrive piattaforma Omeka S, tecnologia IIIF per immagini e visualizzazione con Mirador Viewer. Test live 2026-06-09: item Corbiere 199245 con immagine originale pubblica e manifest https://dl.ficlit.unibo.it/iiif/2/199245/manifest, codice 200 e 1 canvas; item Camporesi 28429 con immagine originale pubblica e manifest https://dl.ficlit.unibo.it/iiif/2/28429/manifest, codice 200 e 239 canvas. Il pattern Omeka/IIIF appare concreto; restano da verificare termini item set e distinzione tra collezioni liberamente scaricabili e sola consultazione</x:v>
       </x:c>
-      <x:c r="G20" s="10" t="str">
+      <x:c r="G21" s="10" t="str">
         <x:v>A - promosso a supporto tecnico R_LIMITED: solo item/manifest FICLIT pubblici, range esplicito, referer FICLIT e verifica termini item-level</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="1320" hidden="0" customHeight="1">
-      <x:c r="A21" s="10" t="str">
+    <x:row r="22" ht="1584" hidden="0" customHeight="1">
+      <x:c r="A22" s="10" t="str">
         <x:v>impronte_digitali_unifi</x:v>
       </x:c>
-      <x:c r="B21" s="10" t="str">
+      <x:c r="B22" s="10" t="str">
         <x:v>Impronte Digitali / Universita di Firenze</x:v>
       </x:c>
-      <x:c r="C21" s="10" t="str">
+      <x:c r="C22" s="10" t="str">
         <x:v>Italia / Toscana</x:v>
       </x:c>
-      <x:c r="D21" s="10" t="str">
+      <x:c r="D22" s="10" t="str">
         <x:v>https://improntedigitali.unifi.it/; news ufficiale https://www.sba.unifi.it/n2411.html; collezioni digitalizzate https://www.sba.unifi.it/p1308.html; campione https://improntedigitali.unifi.it/items/ea8510d3-4f09-41b6-b69a-5c4ff3d0d082; sonda verify_unifi_technical_probe.py</x:v>
       </x:c>
-      <x:c r="E21" s="10" t="str">
+      <x:c r="E22" s="10" t="str">
         <x:v>Media-alta: periodici, fondi archivistici, materiali rari e di pregio delle biblioteche Unifi, con interesse per contesto storico toscano e universitario</x:v>
       </x:c>
-      <x:c r="F21" s="10" t="str">
+      <x:c r="F22" s="10" t="str">
         <x:v>Controllo 2026-07-26 + ricontrollo 2026-07-29: la fonte ufficiale UniFI descrive il portale come digital library pubblica basata su DSpace-GLAM con viewer Mirador e standard IIIF. Verifica live sull'item Ricordi di architettura (ea8510d3-4f09-41b6-b69a-5c4ff3d0d082): API pubblica server/api/core/items/{uuid} leggibile senza login; bundle pubblici ORIGINAL, LICENSE e MAG; metadati item-level con dc.rights.holder UniFI e dc.rights.license = CC BY-NC-SA; file MAG scaricabile con codice 200; thumbnail generato (THUMBNAIL) accessibile come immagine JPEG pubblica, anche via endpoint item-level /thumbnail. Il ricontrollo del 2026-07-29 amplia il quadro del backend pubblico (record, entity correlate, item API, bundle, bitstream e surrogate, 410 candidati classificati), ma non cambia la sostanza: il primo bitstream immagine del bundle ORIGINAL resta 401 sul content diretto, i metadati del bitstream segnalano bitstream.viewer.provider = iiif insieme a nodownload, e non emergono manifest IIIF pubblici espliciti o info.json riusabili</x:v>
       </x:c>
-      <x:c r="G21" s="10" t="str">
+      <x:c r="G22" s="10" t="str">
         <x:v>B - candidato forte e reale per backend DSpace-GLAM/IIIF, confermato in REVIEW: metadata e surrogate web pubblici si', ma senza download/manifest diretto ancora riusabile</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="514.7999877929688" hidden="0" customHeight="1">
-      <x:c r="A22" s="10" t="str">
+    <x:row r="23" ht="1491.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A23" s="10" t="str">
         <x:v>doge_unige</x:v>
       </x:c>
-      <x:c r="B22" s="10" t="str">
+      <x:c r="B23" s="10" t="str">
         <x:v>DOGE Digital Library / Universita di Genova</x:v>
       </x:c>
-      <x:c r="C22" s="10" t="str">
+      <x:c r="C23" s="10" t="str">
         <x:v>Italia / Liguria</x:v>
       </x:c>
-      <x:c r="D22" s="10" t="str">
+      <x:c r="D23" s="10" t="str">
         <x:v>https://doge.unige.net/; fonti SBA https://biblioteche.unige.it/doge_informazioni_generali, https://biblioteche.unige.it/doge_servizi_offerti; campione https://doge.unige.net/entities/publication/b1c2be2c-e1ae-4676-93e3-07e8e8398f72; sonda verify_doge_technical_probe.py</x:v>
       </x:c>
-      <x:c r="E22" s="10" t="str">
+      <x:c r="E23" s="10" t="str">
         <x:v>Media-alta: libri antichi, materiali scientifici, disegni, fondi storici e patrimonio universitario ligure, utile per contesto storico territoriale e bibliografico</x:v>
       </x:c>
-      <x:c r="F22" s="10" t="str">
+      <x:c r="F23" s="10" t="str">
         <x:v>Controllo 2026-07-26/27: le fonti ufficiali SBA descrivono DOGE come digital library basata su DSpace-GLAM, con Mirador, protocollo IIIF, OAI-PMH e licenza generale CC BY-SA per gli oggetti UniGe, CC0 per i metadati. Verifica live sul campione Euler b1c2be2c-e1ae-4676-93e3-07e8e8398f72: item API pubblico, handle persistente, dc.rights.license = CC BY-SA; bundle ORIGINAL, THUMBNAIL, BRANDED_PREVIEW, IIIF-PDF-*, IIIF-ALTERNATIVE-LD e IIIF-ALTERNATIVE-DOWNLOAD. I contenuti ORIGINAL e IIIF-PDF-* restano bloccati o marcati nodownload, ma i derivati IIIF-ALTERNATIVE-LD risultano pubblici pagina-per-pagina con 373 bitstream JPEG numerati e IIIF-ALTERNATIVE-DOWNLOAD espone un PDF derivato pubblico con codice 200. ATK-Pro ora costruisce quindi un manifest sintetico prudente solo dai derivati IIIF-ALTERNATIVE-LD, con PDF derivato in seeAlso, referer DOGE, range esplicito e senza toccare originali o frame viewer nodownload</x:v>
       </x:c>
-      <x:c r="G22" s="10" t="str">
+      <x:c r="G23" s="10" t="str">
         <x:v>A - promosso a supporto tecnico prudente R_LIMITED: solo derivati pubblici IIIF-ALTERNATIVE-LD + IIIF-ALTERNATIVE-DOWNLOAD, con controllo licenza item-level e divieto di estensione agli originali</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="501.6000061035156" hidden="0" customHeight="1">
-      <x:c r="A23" s="10" t="str">
+    <x:row r="24" ht="1320" hidden="0" customHeight="1">
+      <x:c r="A24" s="10" t="str">
         <x:v>orientales_unior</x:v>
       </x:c>
-      <x:c r="B23" s="10" t="str">
+      <x:c r="B24" s="10" t="str">
         <x:v>OrienTales / Biblioteca digitale Universita di Napoli L'Orientale</x:v>
       </x:c>
-      <x:c r="C23" s="10" t="str">
+      <x:c r="C24" s="10" t="str">
         <x:v>Italia / Campania</x:v>
       </x:c>
-      <x:c r="D23" s="10" t="str">
+      <x:c r="D24" s="10" t="str">
         <x:v>https://www.unior.it/it/biblioteche/servizi-gli-utenti/biblioteca-digitale</x:v>
       </x:c>
-      <x:c r="E23" s="10" t="str">
+      <x:c r="E24" s="10" t="str">
         <x:v>Media-alta: libri antichi, manoscritti in lingue orientali, materiale d'archivio, documentario, periodici, collane, carte geografiche e atlanti, con valore culturale e storico per ricerche italiane</x:v>
       </x:c>
-      <x:c r="F23" s="10" t="str">
+      <x:c r="F24" s="10" t="str">
         <x:v>Controllo 2026-06-08/10: fonte ufficiale indica licenze Creative Commons, framework IIIF, uso di Mirador, download laddove la licenza lo permetta, OCR e scarico metadati; la descrizione tecnica cita DSpace, mentre restano possibili tracce Omeka dai progetti precedenti. verify_orientales_technical_probe.py ora cerca sia pattern DSpace (entities, REST item, bundle, bitstream, handle e link JSON/HAL), sia record Omeka, viewer Mirador, manifest IIIF, info.json, immagini, OCR/testi e metadati candidati. Verifica manuale 2026-06-10: le pagine record finora viste mostrano "Il record non puo essere mostrato agli utenti ospiti" e contenuti riservati agli utenti affiliati; manca quindi il requisito minimo di accesso pubblico senza autenticazione. Il download non e generalizzabile senza record pubblici e licenza dell'oggetto</x:v>
       </x:c>
-      <x:c r="G23" s="10" t="str">
+      <x:c r="G24" s="10" t="str">
         <x:v>C - sospeso/escluso dal download automatico finche non emergono record pubblici consultabili da ospite con licenza visibile e endpoint manifest/bitstream senza autenticazione</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="660" hidden="0" customHeight="1">
-      <x:c r="A24" s="10" t="str">
+    <x:row r="25" ht="514.7999877929688" hidden="0" customHeight="1">
+      <x:c r="A25" s="10" t="str">
         <x:v>museu_imigracao_sp</x:v>
       </x:c>
-      <x:c r="B24" s="10" t="str">
+      <x:c r="B25" s="10" t="str">
         <x:v>Museu da Imigracao do Estado de Sao Paulo - Acervo Digital</x:v>
-      </x:c>
-      <x:c r="C24" s="10" t="str">
-        <x:v>Brasile / diaspora italiana</x:v>
-      </x:c>
-      <x:c r="D24" s="10" t="str">
-        <x:v>https://museudaimigracao.org.br/acervo/sobre-acervo; https://www.museudaimigracao.org.br/acervo/passageiros; https://museudaimigracao.org.br/acervo-e-pesquisa/acervo</x:v>
-      </x:c>
-      <x:c r="E24" s="10" t="str">
-        <x:v>Molto alta per immigrati italiani in Brasile/Sao Paulo</x:v>
-      </x:c>
-      <x:c r="F24" s="10" t="str">
-        <x:v>Acervo digitale pubblico con piu di 250 mila immagini, registri di matricola, liste di bordo, carte di chiamata, richieste SACOP, iconografie, cartografie e giornali; le fonti ufficiali indicano uso/download non commerciale, ma il percorso tecnico appare basato su ricerca web e PDF/immagini pubbliche, non su IIIF/API documentata</x:v>
-      </x:c>
-      <x:c r="G24" s="10" t="str">
-        <x:v>B - candidato forte, ma non integrare finche non viene validata una capability pdf_direct/download diretto pubblica e testabile</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="633.5999755859375" hidden="0" customHeight="1">
-      <x:c r="A25" s="10" t="str">
-        <x:v>apesp_digitalizados</x:v>
-      </x:c>
-      <x:c r="B25" s="10" t="str">
-        <x:v>Arquivo Publico do Estado de Sao Paulo - Acervo digitalizado</x:v>
       </x:c>
       <x:c r="C25" s="10" t="str">
         <x:v>Brasile / diaspora italiana</x:v>
       </x:c>
       <x:c r="D25" s="10" t="str">
-        <x:v>https://web.arquivoestado.sp.gov.br/web/acervo/digitalizados; https://www.arquivoestado.sp.gov.br/web/digitalizado/textual/nucleos_coloniais; https://web.arquivoestado.sp.gov.br/web/acervo/atendimento/reproducao_documentos; https://web.arquivoestado.sp.gov.br/web/acervo/solicitacao_certidoes/imigracao</x:v>
+        <x:v>https://museudaimigracao.org.br/acervo/sobre-acervo; https://www.museudaimigracao.org.br/acervo/passageiros; https://museudaimigracao.org.br/acervo-e-pesquisa/acervo</x:v>
       </x:c>
       <x:c r="E25" s="10" t="str">
-        <x:v>Molto alta: Hospedaria, Porto di Santos, nuclei coloniali, documenti di immigrazione e colonizzazione</x:v>
+        <x:v>Molto alta per immigrati italiani in Brasile/Sao Paulo</x:v>
       </x:c>
       <x:c r="F25" s="10" t="str">
-        <x:v>Fonte ufficiale molto rilevante, ma l'acervo digitalizzato rimanda a registrazione/login e la pagina dei nuclei coloniali contiene avviso di servizio con login; la riproduzione e soggetta a credito, termini di responsabilita e valutazioni su diritto/autorizzazione. Nessun endpoint no-login/API/IIIF stabile verificato nel primo controllo</x:v>
+        <x:v>Acervo digitale pubblico con piu di 250 mila immagini, registri di matricola, liste di bordo, carte di chiamata, richieste SACOP, iconografie, cartografie e giornali; le fonti ufficiali indicano uso/download non commerciale, ma il percorso tecnico appare basato su ricerca web e PDF/immagini pubbliche, non su IIIF/API documentata</x:v>
       </x:c>
       <x:c r="G25" s="10" t="str">
-        <x:v>C - link/manuale e discovery; download diretto escluso finche non emerge una risorsa pubblica no-login con licenza e tecnica stabili</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="607.2000122070312" hidden="0" customHeight="1">
+        <x:v>B - candidato forte, ma non integrare finche non viene validata una capability pdf_direct/download diretto pubblica e testabile</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="501.6000061035156" hidden="0" customHeight="1">
       <x:c r="A26" s="10" t="str">
-        <x:v>arquivo_nacional_br_sian</x:v>
+        <x:v>apesp_digitalizados</x:v>
       </x:c>
       <x:c r="B26" s="10" t="str">
-        <x:v>Arquivo Nacional do Brasil / SIAN</x:v>
+        <x:v>Arquivo Publico do Estado de Sao Paulo - Acervo digitalizado</x:v>
       </x:c>
       <x:c r="C26" s="10" t="str">
         <x:v>Brasile / diaspora italiana</x:v>
       </x:c>
       <x:c r="D26" s="10" t="str">
+        <x:v>https://web.arquivoestado.sp.gov.br/web/acervo/digitalizados; https://www.arquivoestado.sp.gov.br/web/digitalizado/textual/nucleos_coloniais; https://web.arquivoestado.sp.gov.br/web/acervo/atendimento/reproducao_documentos; https://web.arquivoestado.sp.gov.br/web/acervo/solicitacao_certidoes/imigracao</x:v>
+      </x:c>
+      <x:c r="E26" s="10" t="str">
+        <x:v>Molto alta: Hospedaria, Porto di Santos, nuclei coloniali, documenti di immigrazione e colonizzazione</x:v>
+      </x:c>
+      <x:c r="F26" s="10" t="str">
+        <x:v>Fonte ufficiale molto rilevante, ma l'acervo digitalizzato rimanda a registrazione/login e la pagina dei nuclei coloniali contiene avviso di servizio con login; la riproduzione e soggetta a credito, termini di responsabilita e valutazioni su diritto/autorizzazione. Nessun endpoint no-login/API/IIIF stabile verificato nel primo controllo</x:v>
+      </x:c>
+      <x:c r="G26" s="10" t="str">
+        <x:v>C - link/manuale e discovery; download diretto escluso finche non emerge una risorsa pubblica no-login con licenza e tecnica stabili</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="660" hidden="0" customHeight="1">
+      <x:c r="A27" s="10" t="str">
+        <x:v>arquivo_nacional_br_sian</x:v>
+      </x:c>
+      <x:c r="B27" s="10" t="str">
+        <x:v>Arquivo Nacional do Brasil / SIAN</x:v>
+      </x:c>
+      <x:c r="C27" s="10" t="str">
+        <x:v>Brasile / diaspora italiana</x:v>
+      </x:c>
+      <x:c r="D27" s="10" t="str">
         <x:v>https://www.gov.br/arquivonacional/pt-br/canais_atendimento/imprensa/copy_of_noticias/a-imigracao-italiana-e-o-acervo-do-an; https://www.gov.br/arquivonacional/pt-br/canais_atendimento/imprensa/copy_of_noticias/quer-pesquisar-no-arquivo-nacional-acesse-o-sian; https://www.gov.br/arquivonacional/pt-br/servicos/acervos/copy_of_acervos-mais-consultados/entrada-de-estrangeiros; https://www.gov.br/arquivonacional/pt-br/servicos/bases-de-dados/bases</x:v>
       </x:c>
-      <x:c r="E26" s="10" t="str">
+      <x:c r="E27" s="10" t="str">
         <x:v>Alta: ingresso di stranieri, vapori, acervo nazionale, Porto di Rio de Janeiro e Porto di Santos</x:v>
       </x:c>
-      <x:c r="F26" s="10" t="str">
+      <x:c r="F27" s="10" t="str">
         <x:v>SIAN e molto rilevante e offre documenti digitalizzati senza costo, ma le fonti ufficiali richiedono cadastro/login; la pagina SIAN espone anche controllo anti-spam/umano. La base separata Entrada de Estrangeiros - Porto do Rio de Janeiro e utile come ricerca nominale/dichiarazione, ma non e ancora un endpoint immagini/API verificato</x:v>
       </x:c>
-      <x:c r="G26" s="10" t="str">
+      <x:c r="G27" s="10" t="str">
         <x:v>C - link/manuale e discovery; non integrare download diretto SIAN per login/challenge. Rivalutare separatamente la base Rio solo se emerge un accesso pubblico documentato e testabile</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="739.2000122070312" hidden="0" customHeight="1">
-      <x:c r="A27" s="10" t="str">
+    <x:row r="28" ht="633.5999755859375" hidden="0" customHeight="1">
+      <x:c r="A28" s="10" t="str">
         <x:v>agn_argentina_inmigrantes</x:v>
       </x:c>
-      <x:c r="B27" s="10" t="str">
+      <x:c r="B28" s="10" t="str">
         <x:v>Archivo General de la Nacion Argentina - buscador inmigrantes</x:v>
-      </x:c>
-      <x:c r="C27" s="10" t="str">
-        <x:v>Argentina / diaspora italiana</x:v>
-      </x:c>
-      <x:c r="D27" s="10" t="str">
-        <x:v>https://www.argentina.gob.ar/interior/archivo-general-de-la-nacion; https://www.argentina.gob.ar/interior/archivo-general-de-la-nacion/consulta-de-antecedentes-migratorios; https://www.argentina.gob.ar/noticias/el-archivo-general-de-la-nacion-es-memoria-del-mundo; https://www.argentina.gob.ar/terminos-y-condiciones; https://www.unesco.org/es/memory-world/lac/passengers-entry-books-sea-1882-1937-national-registry-migrations-documentary-fond</x:v>
-      </x:c>
-      <x:c r="E27" s="10" t="str">
-        <x:v>Molto alta: ingressi al porto di Buenos Aires 1882-1937, serie UNESCO Memoria del Mundo, oltre 4 milioni di ingressi in 808 libri</x:v>
-      </x:c>
-      <x:c r="F27" s="10" t="str">
-        <x:v>Buscador ufficiale pubblico: la pagina indica ricerca per date, nome, cognome e nave, con possibilita di scaricare una constancia PDF e, se digitalizzato, il PDF del libro completo. I termini generali Argentina.gob.ar indicano accesso libero/gratuito e contenuti CC BY 4.0 salvo diversa indicazione; non emergono pero API/IIIF o endpoint ufficiali documentati per automazione</x:v>
-      </x:c>
-      <x:c r="G27" s="10" t="str">
-        <x:v>B - candidato forte per futura capability metadata/PDF; per ora link assistito, no download diretto finche non viene validato un endpoint pubblico stabile con fixture</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="158.39999389648438" hidden="0" customHeight="1">
-      <x:c r="A28" s="10" t="str">
-        <x:v>cemla_buscador</x:v>
-      </x:c>
-      <x:c r="B28" s="10" t="str">
-        <x:v>CEMLA buscador inmigrantes</x:v>
       </x:c>
       <x:c r="C28" s="10" t="str">
         <x:v>Argentina / diaspora italiana</x:v>
       </x:c>
       <x:c r="D28" s="10" t="str">
+        <x:v>https://www.argentina.gob.ar/interior/archivo-general-de-la-nacion; https://www.argentina.gob.ar/interior/archivo-general-de-la-nacion/consulta-de-antecedentes-migratorios; https://www.argentina.gob.ar/noticias/el-archivo-general-de-la-nacion-es-memoria-del-mundo; https://www.argentina.gob.ar/terminos-y-condiciones; https://www.unesco.org/es/memory-world/lac/passengers-entry-books-sea-1882-1937-national-registry-migrations-documentary-fond</x:v>
+      </x:c>
+      <x:c r="E28" s="10" t="str">
+        <x:v>Molto alta: ingressi al porto di Buenos Aires 1882-1937, serie UNESCO Memoria del Mundo, oltre 4 milioni di ingressi in 808 libri</x:v>
+      </x:c>
+      <x:c r="F28" s="10" t="str">
+        <x:v>Buscador ufficiale pubblico: la pagina indica ricerca per date, nome, cognome e nave, con possibilita di scaricare una constancia PDF e, se digitalizzato, il PDF del libro completo. I termini generali Argentina.gob.ar indicano accesso libero/gratuito e contenuti CC BY 4.0 salvo diversa indicazione; non emergono pero API/IIIF o endpoint ufficiali documentati per automazione</x:v>
+      </x:c>
+      <x:c r="G28" s="10" t="str">
+        <x:v>B - candidato forte per futura capability metadata/PDF; per ora link assistito, no download diretto finche non viene validato un endpoint pubblico stabile con fixture</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="607.2000122070312" hidden="0" customHeight="1">
+      <x:c r="A29" s="10" t="str">
+        <x:v>cemla_buscador</x:v>
+      </x:c>
+      <x:c r="B29" s="10" t="str">
+        <x:v>CEMLA buscador inmigrantes</x:v>
+      </x:c>
+      <x:c r="C29" s="10" t="str">
+        <x:v>Argentina / diaspora italiana</x:v>
+      </x:c>
+      <x:c r="D29" s="10" t="str">
         <x:v>https://cemla.com/; https://www.cemla.com/buscador/; https://cemla.com/faqs/; https://cemla.com/contacto/; https://cemla.com/terms-and-conditions/</x:v>
       </x:c>
-      <x:c r="E28" s="10" t="str">
+      <x:c r="E29" s="10" t="str">
         <x:v>Alta: arrivi di immigrati in Argentina, con dati fino al 1960 e forte utilita per famiglie italiane</x:v>
       </x:c>
-      <x:c r="F28" s="10" t="str">
+      <x:c r="F29" s="10" t="str">
         <x:v>Fonte privata/non governativa molto usata; le FAQ chiariscono che CEMLA espone solo i dati presenti nel buscador, indica i campi disponibili e rimanda al certificato via email. Il buscador e incorporato come iframe, non espone API/IIIF o endpoint documentati, la pagina termini e un placeholder generico e il flusso pubblico richiede validazione tipo CAPTCHA</x:v>
       </x:c>
-      <x:c r="G28" s="10" t="str">
+      <x:c r="G29" s="10" t="str">
         <x:v>C - solo link/manuale; no download diretto e no interrogazione automatica senza autorizzazione/API esplicita</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="158.39999389648438" hidden="0" customHeight="1">
-      <x:c r="A29" s="10" t="str">
+    <x:row r="30" ht="739.2000122070312" hidden="0" customHeight="1">
+      <x:c r="A30" s="10" t="str">
         <x:v>agn_colombia_dataviva</x:v>
       </x:c>
-      <x:c r="B29" s="10" t="str">
+      <x:c r="B30" s="10" t="str">
         <x:v>Archivo General de la Nacion Colombia - DataViva</x:v>
       </x:c>
-      <x:c r="C29" s="10" t="str">
+      <x:c r="C30" s="10" t="str">
         <x:v>Colombia / diaspora italiana</x:v>
       </x:c>
-      <x:c r="D29" s="10" t="str">
+      <x:c r="D30" s="10" t="str">
         <x:v>https://www.archivogeneral.gov.co/agn/home/; https://dataviva.archivogeneral.gov.co/; https://www.datos.gov.co/Cultura/DATAVIVA/r5h9-7h58; https://www.archivogeneral.gov.co/dataviva-da-un-paso-historico-hacia-los-datos-abiertos-en-colombia; https://www.archivogeneral.gov.co/terminos-y-condiciones; https://www.archivogeneral.gov.co/sites/default/files/2025-07/MANUAL_DATAVIVA.pdf</x:v>
       </x:c>
-      <x:c r="E29" s="10" t="str">
+      <x:c r="E30" s="10" t="str">
         <x:v>Media-alta: documenti storici digitalizzati, possibili fondi migrazione e contesto per presenze italiane in Colombia</x:v>
       </x:c>
-      <x:c r="F29" s="10" t="str">
+      <x:c r="F30" s="10" t="str">
         <x:v>Candidato tecnico forte per metadata/discovery: il dataset ufficiale Datos Abiertos Colombia dichiara DataViva come applicazione AGN per consulta, visualizzazione e descarga di piu di 25 milioni di immagini, con accesso OData/Socrata e dati aggiornati nel 2026. Tuttavia i termini generali AGN sono restrittivi su riproduzione/copia/distribuzione dei contenuti; distinguere metadati open data da immagini/documenti e verificare per item prima di qualunque download</x:v>
       </x:c>
-      <x:c r="G29" s="10" t="str">
+      <x:c r="G30" s="10" t="str">
         <x:v>B - forte per futura integrazione metadata/API; download immagini/PDF solo con policy specifica, range esplicito e fixture stabile</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="132" hidden="0" customHeight="1">
-      <x:c r="A30" s="10" t="str">
+    <x:row r="31" ht="158.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A31" s="10" t="str">
         <x:v>nara_catalog</x:v>
       </x:c>
-      <x:c r="B30" s="10" t="str">
+      <x:c r="B31" s="10" t="str">
         <x:v>National Archives Catalog / NARA API</x:v>
       </x:c>
-      <x:c r="C30" s="10" t="str">
+      <x:c r="C31" s="10" t="str">
         <x:v>Stati Uniti / diaspora italiana</x:v>
       </x:c>
-      <x:c r="D30" s="10" t="str">
+      <x:c r="D31" s="10" t="str">
         <x:v>https://www.archives.gov/research/catalog/help/api; https://www.archives.gov/research/immigration/overview</x:v>
       </x:c>
-      <x:c r="E30" s="10" t="str">
+      <x:c r="E31" s="10" t="str">
         <x:v>Alta: naturalizzazioni, immigrazione, passenger records, A-files</x:v>
       </x:c>
-      <x:c r="F30" s="10" t="str">
+      <x:c r="F31" s="10" t="str">
         <x:v>API ufficiale per dati pubblici del Catalog; disponibilita immagini e diritti variano per record</x:v>
       </x:c>
-      <x:c r="G30" s="10" t="str">
+      <x:c r="G31" s="10" t="str">
         <x:v>A/B - candidato forte per metadata/record pubblici</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="237.60000610351562" hidden="0" customHeight="1">
-      <x:c r="A31" s="10" t="str">
-        <x:v>loc_chronicling_america</x:v>
-      </x:c>
-      <x:c r="B31" s="10" t="str">
-        <x:v>Library of Congress - Chronicling America / loc.gov API</x:v>
-      </x:c>
-      <x:c r="C31" s="10" t="str">
-        <x:v>Stati Uniti / contesto diaspora</x:v>
-      </x:c>
-      <x:c r="D31" s="10" t="str">
-        <x:v>https://www.loc.gov/apis/additional-apis/chronicling-america-api/</x:v>
-      </x:c>
-      <x:c r="E31" s="10" t="str">
-        <x:v>Media: giornali storici utili per contesto familiare, non atti vitali</x:v>
-      </x:c>
-      <x:c r="F31" s="10" t="str">
-        <x:v>API ufficiale; utile come modulo di ricerca contestuale piu che downloader genealogico primario</x:v>
-      </x:c>
-      <x:c r="G31" s="10" t="str">
-        <x:v>B - valutare dopo fonti archivistiche</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A32" s="10" t="str">
+        <x:v>loc_chronicling_america</x:v>
+      </x:c>
+      <x:c r="B32" s="10" t="str">
+        <x:v>Library of Congress - Chronicling America / loc.gov API</x:v>
+      </x:c>
+      <x:c r="C32" s="10" t="str">
+        <x:v>Stati Uniti / contesto diaspora</x:v>
+      </x:c>
+      <x:c r="D32" s="10" t="str">
+        <x:v>https://www.loc.gov/apis/additional-apis/chronicling-america-api/</x:v>
+      </x:c>
+      <x:c r="E32" s="10" t="str">
+        <x:v>Media: giornali storici utili per contesto familiare, non atti vitali</x:v>
+      </x:c>
+      <x:c r="F32" s="10" t="str">
+        <x:v>API ufficiale; utile come modulo di ricerca contestuale piu che downloader genealogico primario</x:v>
+      </x:c>
+      <x:c r="G32" s="10" t="str">
+        <x:v>B - valutare dopo fonti archivistiche</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="132" hidden="0" customHeight="1">
+      <x:c r="A33" s="10" t="str">
         <x:v>naa_recordsearch</x:v>
       </x:c>
-      <x:c r="B32" s="10" t="str">
+      <x:c r="B33" s="10" t="str">
         <x:v>National Archives of Australia - RecordSearch passenger arrivals</x:v>
       </x:c>
-      <x:c r="C32" s="10" t="str">
+      <x:c r="C33" s="10" t="str">
         <x:v>Australia / diaspora italiana</x:v>
       </x:c>
-      <x:c r="D32" s="10" t="str">
+      <x:c r="D33" s="10" t="str">
         <x:v>https://www.naa.gov.au/explore-collection/immigration-and-citizenship/passenger-arrival-records</x:v>
       </x:c>
-      <x:c r="E32" s="10" t="str">
+      <x:c r="E33" s="10" t="str">
         <x:v>Alta: arrivi passeggeri 1898-1972, dati migratori</x:v>
       </x:c>
-      <x:c r="F32" s="10" t="str">
+      <x:c r="F33" s="10" t="str">
         <x:v>Fonte ufficiale e molto rilevante; API non confermata, diritti/download da verificare</x:v>
       </x:c>
-      <x:c r="G32" s="10" t="str">
+      <x:c r="G33" s="10" t="str">
         <x:v>B/C - candidato prioritario, inizialmente link assistito</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="224.39999389648438" hidden="0" customHeight="1">
-      <x:c r="A33" s="10" t="str">
+    <x:row r="34" ht="237.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A34" s="10" t="str">
         <x:v>papers_past_digitalnz</x:v>
       </x:c>
-      <x:c r="B33" s="10" t="str">
+      <x:c r="B34" s="10" t="str">
         <x:v>Papers Past / DigitalNZ API</x:v>
       </x:c>
-      <x:c r="C33" s="10" t="str">
+      <x:c r="C34" s="10" t="str">
         <x:v>Nuova Zelanda / diaspora italiana</x:v>
       </x:c>
-      <x:c r="D33" s="10" t="str">
+      <x:c r="D34" s="10" t="str">
         <x:v>https://natlib.govt.nz/about-us/open-data/papers-past-metadata/papers-past-data-using-the-digitalnz-api; https://paperspast.natlib.govt.nz/help/using-papers-past-material</x:v>
       </x:c>
-      <x:c r="E33" s="10" t="str">
+      <x:c r="E34" s="10" t="str">
         <x:v>Media: giornali e avvisi utili per tracce migratorie e familiari</x:v>
       </x:c>
-      <x:c r="F33" s="10" t="str">
+      <x:c r="F34" s="10" t="str">
         <x:v>API metadata ufficiale via DigitalNZ; immagini/testi e copyright da verificare per item</x:v>
       </x:c>
-      <x:c r="G33" s="10" t="str">
+      <x:c r="G34" s="10" t="str">
         <x:v>B - candidato per ricerca contestuale</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="198" hidden="0" customHeight="1">
-      <x:c r="A34" s="10" t="str">
+    <x:row r="35" ht="158.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A35" s="10" t="str">
         <x:v>francearchives</x:v>
       </x:c>
-      <x:c r="B34" s="10" t="str">
+      <x:c r="B35" s="10" t="str">
         <x:v>FranceArchives open data</x:v>
       </x:c>
-      <x:c r="C34" s="10" t="str">
+      <x:c r="C35" s="10" t="str">
         <x:v>Francia / diaspora italiana</x:v>
       </x:c>
-      <x:c r="D34" s="10" t="str">
+      <x:c r="D35" s="10" t="str">
         <x:v>https://francearchives.gouv.fr/fr/open_data</x:v>
       </x:c>
-      <x:c r="E34" s="10" t="str">
+      <x:c r="E35" s="10" t="str">
         <x:v>Alta per ricerche in Francia e migrazioni confinanti</x:v>
       </x:c>
-      <x:c r="F34" s="10" t="str">
+      <x:c r="F35" s="10" t="str">
         <x:v>Dati aperti e aggregazione di inventari; immagini e archivi dipartimentali dipendono dai provider</x:v>
       </x:c>
-      <x:c r="G34" s="10" t="str">
+      <x:c r="G35" s="10" t="str">
         <x:v>B - ottimo per discovery, download solo per provider verificati</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="211.1999969482422" hidden="0" customHeight="1">
-      <x:c r="A35" s="10" t="str">
+    <x:row r="36" ht="224.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A36" s="10" t="str">
         <x:v>belgium_state_archives</x:v>
       </x:c>
-      <x:c r="B35" s="10" t="str">
+      <x:c r="B36" s="10" t="str">
         <x:v>State Archives of Belgium / AGATHA</x:v>
       </x:c>
-      <x:c r="C35" s="10" t="str">
+      <x:c r="C36" s="10" t="str">
         <x:v>Belgio / diaspora italiana</x:v>
       </x:c>
-      <x:c r="D35" s="10" t="str">
+      <x:c r="D36" s="10" t="str">
         <x:v>https://archives.brussels.be/genealogy; https://news.belgium.be/fr/registres-paroissiaux-et-de-letat-civil-consultables-en-ligne-gratuitement</x:v>
       </x:c>
-      <x:c r="E35" s="10" t="str">
+      <x:c r="E36" s="10" t="str">
         <x:v>Alta: stato civile e registri parrocchiali</x:v>
       </x:c>
-      <x:c r="F35" s="10" t="str">
+      <x:c r="F36" s="10" t="str">
         <x:v>Consultazione gratuita ma storicamente richiede account/login per archivi online; non automatizzare accessi autenticati</x:v>
       </x:c>
-      <x:c r="G35" s="10" t="str">
+      <x:c r="G36" s="10" t="str">
         <x:v>C - link/manuale, no integrazione diretta se login necessario</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="264" hidden="0" customHeight="1">
-      <x:c r="A36" s="10" t="str">
+    <x:row r="37" ht="198" hidden="0" customHeight="1">
+      <x:c r="A37" s="10" t="str">
         <x:v>deutsche_digitale_bibliothek</x:v>
       </x:c>
-      <x:c r="B36" s="10" t="str">
+      <x:c r="B37" s="10" t="str">
         <x:v>Deutsche Digitale Bibliothek / DDB API</x:v>
       </x:c>
-      <x:c r="C36" s="10" t="str">
+      <x:c r="C37" s="10" t="str">
         <x:v>Germania / diaspora italiana</x:v>
       </x:c>
-      <x:c r="D36" s="10" t="str">
+      <x:c r="D37" s="10" t="str">
         <x:v>https://www.deutsche-digitale-bibliothek.de/content/api-nutzungsbedingungen?lang=en; https://labs.deutsche-digitale-bibliothek.de/app/ddbapi/</x:v>
       </x:c>
-      <x:c r="E36" s="10" t="str">
+      <x:c r="E37" s="10" t="str">
         <x:v>Media-alta: aggregatore culturale/archivistico tedesco</x:v>
       </x:c>
-      <x:c r="F36" s="10" t="str">
+      <x:c r="F37" s="10" t="str">
         <x:v>API ufficiale ma richiede API key; diritti e contenuti digitali dipendono dai provider</x:v>
       </x:c>
-      <x:c r="G36" s="10" t="str">
+      <x:c r="G37" s="10" t="str">
         <x:v>B/C - metadata possibile, immagini solo item-by-item</x:v>
       </x:c>
     </x:row>
-    <x:row r="37">
-      <x:c r="A37" t="str">
+    <x:row r="38" ht="211.1999969482422" hidden="0" customHeight="1">
+      <x:c r="A38" s="10" t="str">
         <x:v>austrian_state_archives_ais</x:v>
       </x:c>
-      <x:c r="B37" t="str">
+      <x:c r="B38" s="10" t="str">
         <x:v>Oesterreichisches Staatsarchiv - AIS</x:v>
       </x:c>
-      <x:c r="C37" t="str">
+      <x:c r="C38" s="10" t="str">
         <x:v>Austria / area asburgica</x:v>
       </x:c>
-      <x:c r="D37" t="str">
+      <x:c r="D38" s="10" t="str">
         <x:v>https://www.oesta.gv.at/benutzung/Recherche-zu-Hause/recherche/bestande-ais.html; https://www.statearchives.gv.at/user-information/holdings.html</x:v>
       </x:c>
-      <x:c r="E37" t="str">
+      <x:c r="E38" s="10" t="str">
         <x:v>Alta per Lombardo-Veneto, Trentino-Alto Adige, Friuli Venezia Giulia e fonti militari/asburgiche</x:v>
       </x:c>
-      <x:c r="F37" t="str">
+      <x:c r="F38" s="10" t="str">
         <x:v>Sistema ufficiale di ricerca; utile per discovery e ordinazioni, non ancora candidato downloader</x:v>
       </x:c>
-      <x:c r="G37" t="str">
+      <x:c r="G38" s="10" t="str">
         <x:v>C - link/discovery assistito</x:v>
       </x:c>
     </x:row>
-    <x:row r="38">
-      <x:c r="A38" t="str">
+    <x:row r="39" ht="264" hidden="0" customHeight="1">
+      <x:c r="A39" s="10" t="str">
         <x:v>anno_onb</x:v>
       </x:c>
-      <x:c r="B38" t="str">
+      <x:c r="B39" s="10" t="str">
         <x:v>ANNO - AustriaN Newspapers Online</x:v>
       </x:c>
-      <x:c r="C38" t="str">
+      <x:c r="C39" s="10" t="str">
         <x:v>Austria / area asburgica</x:v>
       </x:c>
-      <x:c r="D38" t="str">
+      <x:c r="D39" s="10" t="str">
         <x:v>https://dbis.ur.de/detail.php?bib_id=FUH&amp;lang=en&amp;titel_id=2012; https://www.bundeskanzleramt.gv.at/en/services/federal-administrative-library/databases/general-access-databases.html</x:v>
       </x:c>
-      <x:c r="E38" t="str">
+      <x:c r="E39" s="10" t="str">
         <x:v>Media: giornali storici per contesto migratorio, militare e civile</x:v>
       </x:c>
-      <x:c r="F38" t="str">
+      <x:c r="F39" s="10" t="str">
         <x:v>Fonte pubblica importante; API ufficiale non confermata nel primo passaggio, evitare scraping massivo</x:v>
       </x:c>
-      <x:c r="G38" t="str">
+      <x:c r="G39" s="10" t="str">
         <x:v>C/B - rivalutare se emerge API stabile o download consentito</x:v>
       </x:c>
     </x:row>

</xml_diff>